<commit_message>
Award fixes (Akers/Jackson) in workbooks
</commit_message>
<xml_diff>
--- a/Trail_Bish_Dynasty_Premium.xlsx
+++ b/Trail_Bish_Dynasty_Premium.xlsx
@@ -884,7 +884,7 @@
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>avg 54.3</t>
+          <t>avg 54.2</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="H4" s="19" t="inlineStr">
         <is>
-          <t>Multiple All-Pro and Pro Bowl cornerback; among the NFL's premier defensive backs; Super Bowl champion.</t>
+          <t>Multiple All-Pro and Pro Bowl cornerback; among the NFL's premier defensive backs.</t>
         </is>
       </c>
     </row>
@@ -1821,25 +1821,25 @@
       </c>
       <c r="B19" s="21" t="inlineStr">
         <is>
-          <t>Ceedee Lamb</t>
+          <t>Micah Parsons</t>
         </is>
       </c>
       <c r="C19" s="22" t="inlineStr">
         <is>
-          <t>WR</t>
-        </is>
-      </c>
-      <c r="D19" s="23" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E19" s="22" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="F19" s="27" t="inlineStr">
         <is>
-          <t>85.5</t>
+          <t>85.1</t>
         </is>
       </c>
       <c r="G19" s="27" t="inlineStr">
@@ -1849,7 +1849,7 @@
       </c>
       <c r="H19" s="25" t="inlineStr">
         <is>
-          <t>Multiple Pro Bowl and All-Pro receiver with several 1,000-yard seasons. [PFR correction — ALL_PRO 0→1.]</t>
+          <t>Multiple All-Pro linebacker and one of the NFL's premier defensive players.</t>
         </is>
       </c>
     </row>
@@ -1859,12 +1859,12 @@
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>Micah Parsons</t>
+          <t>Marlon Humphrey</t>
         </is>
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D20" s="17" t="inlineStr">
@@ -1873,11 +1873,11 @@
         </is>
       </c>
       <c r="E20" s="16" t="n">
-        <v>2021</v>
+        <v>2017</v>
       </c>
       <c r="F20" s="17" t="inlineStr">
         <is>
-          <t>85.1</t>
+          <t>85.0</t>
         </is>
       </c>
       <c r="G20" s="17" t="inlineStr">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="H20" s="19" t="inlineStr">
         <is>
-          <t>Multiple All-Pro linebacker and one of the NFL's premier defensive players.</t>
+          <t>Multiple Pro Bowl and All-Pro cornerback; cornerstone of the Ravens secondary.</t>
         </is>
       </c>
     </row>
@@ -1897,17 +1897,17 @@
       </c>
       <c r="B21" s="21" t="inlineStr">
         <is>
-          <t>Marlon Humphrey</t>
+          <t>Budda Baker</t>
         </is>
       </c>
       <c r="C21" s="22" t="inlineStr">
         <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="D21" s="27" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>FS</t>
+        </is>
+      </c>
+      <c r="D21" s="23" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E21" s="22" t="n">
@@ -1925,7 +1925,7 @@
       </c>
       <c r="H21" s="25" t="inlineStr">
         <is>
-          <t>Multiple Pro Bowl and All-Pro cornerback; cornerstone of the Ravens secondary.</t>
+          <t>Multiple All-Pro and Pro Bowl safety; cornerstone defensive player.</t>
         </is>
       </c>
     </row>
@@ -1935,12 +1935,12 @@
       </c>
       <c r="B22" s="15" t="inlineStr">
         <is>
-          <t>Budda Baker</t>
+          <t>Chris Lindstrom</t>
         </is>
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>FS</t>
+          <t>OL</t>
         </is>
       </c>
       <c r="D22" s="26" t="inlineStr">
@@ -1949,11 +1949,11 @@
         </is>
       </c>
       <c r="E22" s="16" t="n">
-        <v>2017</v>
+        <v>2019</v>
       </c>
       <c r="F22" s="17" t="inlineStr">
         <is>
-          <t>85.0</t>
+          <t>84.0</t>
         </is>
       </c>
       <c r="G22" s="17" t="inlineStr">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="H22" s="19" t="inlineStr">
         <is>
-          <t>Multiple All-Pro and Pro Bowl safety; cornerstone defensive player.</t>
+          <t>Multiple All-Pro and Pro Bowl guard; among the NFL's premier interior linemen.</t>
         </is>
       </c>
     </row>
@@ -1973,12 +1973,12 @@
       </c>
       <c r="B23" s="21" t="inlineStr">
         <is>
-          <t>Chris Lindstrom</t>
+          <t>Ceedee Lamb</t>
         </is>
       </c>
       <c r="C23" s="22" t="inlineStr">
         <is>
-          <t>OL</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D23" s="23" t="inlineStr">
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="E23" s="22" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="F23" s="27" t="inlineStr">
         <is>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="H23" s="25" t="inlineStr">
         <is>
-          <t>Multiple All-Pro and Pro Bowl guard; among the NFL's premier interior linemen.</t>
+          <t>Multiple Pro Bowl and All-Pro receiver with several 1,000-yard seasons.</t>
         </is>
       </c>
     </row>
@@ -2011,12 +2011,12 @@
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>Ja'marr Chase</t>
+          <t>Sauce Gardner</t>
         </is>
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D24" s="26" t="inlineStr">
@@ -2025,7 +2025,7 @@
         </is>
       </c>
       <c r="E24" s="16" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="F24" s="17" t="inlineStr">
         <is>
@@ -2039,7 +2039,7 @@
       </c>
       <c r="H24" s="19" t="inlineStr">
         <is>
-          <t>Multiple Pro Bowl and All-Pro receiver; among the league's most productive pass catchers. [PFR correction — OROY 0→1; ALL_PRO 0→2.]</t>
+          <t>Multiple All-Pro cornerback and one of the NFL's premier coverage defenders.</t>
         </is>
       </c>
     </row>
@@ -2049,25 +2049,25 @@
       </c>
       <c r="B25" s="21" t="inlineStr">
         <is>
-          <t>Sauce Gardner</t>
+          <t>Ryan Ramczyk</t>
         </is>
       </c>
       <c r="C25" s="22" t="inlineStr">
         <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="D25" s="23" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="D25" s="27" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E25" s="22" t="n">
-        <v>2022</v>
+        <v>2017</v>
       </c>
       <c r="F25" s="27" t="inlineStr">
         <is>
-          <t>83.6</t>
+          <t>83.5</t>
         </is>
       </c>
       <c r="G25" s="27" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="H25" s="25" t="inlineStr">
         <is>
-          <t>Multiple All-Pro cornerback and one of the NFL's premier coverage defenders.</t>
+          <t>Multiple All-Pro and Pro Bowl offensive tackle; cornerstone of the Saints offensive line.</t>
         </is>
       </c>
     </row>
@@ -2087,25 +2087,25 @@
       </c>
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>Ryan Ramczyk</t>
+          <t>Joey Bosa</t>
         </is>
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>OT</t>
-        </is>
-      </c>
-      <c r="D26" s="17" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D26" s="26" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E26" s="16" t="n">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="F26" s="17" t="inlineStr">
         <is>
-          <t>83.5</t>
+          <t>82.6</t>
         </is>
       </c>
       <c r="G26" s="17" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="H26" s="19" t="inlineStr">
         <is>
-          <t>Multiple All-Pro and Pro Bowl offensive tackle; cornerstone of the Saints offensive line.</t>
+          <t>Multiple Pro Bowl pass rusher with over 70 career sacks.</t>
         </is>
       </c>
     </row>
@@ -2125,12 +2125,12 @@
       </c>
       <c r="B27" s="21" t="inlineStr">
         <is>
-          <t>Joey Bosa</t>
+          <t>Marshon Lattimore</t>
         </is>
       </c>
       <c r="C27" s="22" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D27" s="23" t="inlineStr">
@@ -2139,7 +2139,7 @@
         </is>
       </c>
       <c r="E27" s="22" t="n">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="F27" s="27" t="inlineStr">
         <is>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="H27" s="25" t="inlineStr">
         <is>
-          <t>Multiple Pro Bowl pass rusher with over 70 career sacks.</t>
+          <t>DROY winner and multiple Pro Bowl cornerback.</t>
         </is>
       </c>
     </row>
@@ -2163,12 +2163,12 @@
       </c>
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>Marshon Lattimore</t>
+          <t>Roquan Smith</t>
         </is>
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>ILB</t>
         </is>
       </c>
       <c r="D28" s="26" t="inlineStr">
@@ -2177,11 +2177,11 @@
         </is>
       </c>
       <c r="E28" s="16" t="n">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="F28" s="17" t="inlineStr">
         <is>
-          <t>82.6</t>
+          <t>82.5</t>
         </is>
       </c>
       <c r="G28" s="17" t="inlineStr">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="H28" s="19" t="inlineStr">
         <is>
-          <t>DROY winner and multiple Pro Bowl cornerback.</t>
+          <t>Multiple All-Pro linebacker and one of the NFL's leading tacklers.</t>
         </is>
       </c>
     </row>
@@ -2201,12 +2201,12 @@
       </c>
       <c r="B29" s="21" t="inlineStr">
         <is>
-          <t>Roquan Smith</t>
+          <t>Amari Cooper</t>
         </is>
       </c>
       <c r="C29" s="22" t="inlineStr">
         <is>
-          <t>ILB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D29" s="23" t="inlineStr">
@@ -2215,11 +2215,11 @@
         </is>
       </c>
       <c r="E29" s="22" t="n">
-        <v>2018</v>
+        <v>2015</v>
       </c>
       <c r="F29" s="27" t="inlineStr">
         <is>
-          <t>82.5</t>
+          <t>82.0</t>
         </is>
       </c>
       <c r="G29" s="27" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="H29" s="25" t="inlineStr">
         <is>
-          <t>Multiple All-Pro linebacker and one of the NFL's leading tacklers.</t>
+          <t>Multiple Pro Bowl receiver with seven 1,000-yard receiving seasons.</t>
         </is>
       </c>
     </row>
@@ -2239,12 +2239,12 @@
       </c>
       <c r="B30" s="15" t="inlineStr">
         <is>
-          <t>Amari Cooper</t>
+          <t>Laremy Tunsil</t>
         </is>
       </c>
       <c r="C30" s="16" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>OT</t>
         </is>
       </c>
       <c r="D30" s="26" t="inlineStr">
@@ -2253,7 +2253,7 @@
         </is>
       </c>
       <c r="E30" s="16" t="n">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="F30" s="17" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="H30" s="19" t="inlineStr">
         <is>
-          <t>Multiple Pro Bowl receiver with seven 1,000-yard receiving seasons.</t>
+          <t>Multiple All-Pro and Pro Bowl offensive tackle; among the league's premier pass protectors.</t>
         </is>
       </c>
     </row>
@@ -2277,21 +2277,21 @@
       </c>
       <c r="B31" s="21" t="inlineStr">
         <is>
-          <t>Laremy Tunsil</t>
+          <t>Jonathan Allen</t>
         </is>
       </c>
       <c r="C31" s="22" t="inlineStr">
         <is>
-          <t>OT</t>
-        </is>
-      </c>
-      <c r="D31" s="23" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D31" s="27" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E31" s="22" t="n">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="F31" s="27" t="inlineStr">
         <is>
@@ -2305,7 +2305,7 @@
       </c>
       <c r="H31" s="25" t="inlineStr">
         <is>
-          <t>Multiple All-Pro and Pro Bowl offensive tackle; among the league's premier pass protectors.</t>
+          <t>Multiple Pro Bowl defensive lineman and key contributor on playoff teams.</t>
         </is>
       </c>
     </row>
@@ -2315,17 +2315,17 @@
       </c>
       <c r="B32" s="15" t="inlineStr">
         <is>
-          <t>Jonathan Allen</t>
+          <t>Leonard Fournette</t>
         </is>
       </c>
       <c r="C32" s="16" t="inlineStr">
         <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D32" s="17" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>RB</t>
+        </is>
+      </c>
+      <c r="D32" s="26" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E32" s="16" t="n">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="F32" s="17" t="inlineStr">
         <is>
-          <t>82.0</t>
+          <t>81.5</t>
         </is>
       </c>
       <c r="G32" s="17" t="inlineStr">
@@ -2343,7 +2343,7 @@
       </c>
       <c r="H32" s="19" t="inlineStr">
         <is>
-          <t>Multiple Pro Bowl defensive lineman and key contributor on playoff teams.</t>
+          <t>Pro Bowl running back and Super Bowl champion with multiple 1,000-yard seasons.</t>
         </is>
       </c>
     </row>
@@ -2353,12 +2353,12 @@
       </c>
       <c r="B33" s="21" t="inlineStr">
         <is>
-          <t>Leonard Fournette</t>
+          <t>Jalen Carter</t>
         </is>
       </c>
       <c r="C33" s="22" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D33" s="23" t="inlineStr">
@@ -2367,7 +2367,7 @@
         </is>
       </c>
       <c r="E33" s="22" t="n">
-        <v>2017</v>
+        <v>2023</v>
       </c>
       <c r="F33" s="27" t="inlineStr">
         <is>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="H33" s="25" t="inlineStr">
         <is>
-          <t>Pro Bowl running back and Super Bowl champion with multiple 1,000-yard seasons.</t>
+          <t>Pro Bowl defensive tackle and key contributor on elite defenses.</t>
         </is>
       </c>
     </row>
@@ -2391,12 +2391,12 @@
       </c>
       <c r="B34" s="15" t="inlineStr">
         <is>
-          <t>Jalen Carter</t>
+          <t>Andrew Luck</t>
         </is>
       </c>
       <c r="C34" s="16" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D34" s="26" t="inlineStr">
@@ -2405,11 +2405,11 @@
         </is>
       </c>
       <c r="E34" s="16" t="n">
-        <v>2023</v>
+        <v>2012</v>
       </c>
       <c r="F34" s="17" t="inlineStr">
         <is>
-          <t>81.5</t>
+          <t>80.0</t>
         </is>
       </c>
       <c r="G34" s="17" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="H34" s="19" t="inlineStr">
         <is>
-          <t>Pro Bowl defensive tackle and key contributor on elite defenses; Super Bowl champion.</t>
+          <t>Four-time Pro Bowl franchise QB with multiple elite seasons and major organizational impact.</t>
         </is>
       </c>
     </row>
@@ -2429,12 +2429,12 @@
       </c>
       <c r="B35" s="21" t="inlineStr">
         <is>
-          <t>Andrew Luck</t>
+          <t>Ja'marr Chase</t>
         </is>
       </c>
       <c r="C35" s="22" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D35" s="23" t="inlineStr">
@@ -2443,7 +2443,7 @@
         </is>
       </c>
       <c r="E35" s="22" t="n">
-        <v>2012</v>
+        <v>2021</v>
       </c>
       <c r="F35" s="27" t="inlineStr">
         <is>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="H35" s="25" t="inlineStr">
         <is>
-          <t>Four-time Pro Bowl franchise QB with multiple elite seasons and major organizational impact.</t>
+          <t>Multiple Pro Bowl and All-Pro receiver; among the league's most productive pass catchers.</t>
         </is>
       </c>
     </row>
@@ -3075,17 +3075,17 @@
       </c>
       <c r="B52" s="15" t="inlineStr">
         <is>
-          <t>Melvin Gordon</t>
+          <t>Leonard Williams</t>
         </is>
       </c>
       <c r="C52" s="16" t="inlineStr">
         <is>
-          <t>RB</t>
-        </is>
-      </c>
-      <c r="D52" s="17" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="D52" s="26" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E52" s="16" t="n">
@@ -3103,7 +3103,7 @@
       </c>
       <c r="H52" s="19" t="inlineStr">
         <is>
-          <t>Multiple Pro Bowl running back with over 6,000 career rushing yards; Super Bowl champion. [PFR correction — SB Win 0→1.]</t>
+          <t>Multiple Pro Bowl defensive lineman with over 70 career sacks.</t>
         </is>
       </c>
     </row>
@@ -3113,21 +3113,21 @@
       </c>
       <c r="B53" s="21" t="inlineStr">
         <is>
-          <t>Leonard Williams</t>
+          <t>Ronnie Stanley</t>
         </is>
       </c>
       <c r="C53" s="22" t="inlineStr">
         <is>
-          <t>DT</t>
-        </is>
-      </c>
-      <c r="D53" s="23" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="D53" s="27" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E53" s="22" t="n">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="F53" s="29" t="inlineStr">
         <is>
@@ -3141,7 +3141,7 @@
       </c>
       <c r="H53" s="25" t="inlineStr">
         <is>
-          <t>Multiple Pro Bowl defensive lineman with over 70 career sacks; Super Bowl champion.</t>
+          <t>Multiple All-Pro and Pro Bowl offensive tackle; cornerstone left tackle.</t>
         </is>
       </c>
     </row>
@@ -3151,17 +3151,17 @@
       </c>
       <c r="B54" s="15" t="inlineStr">
         <is>
-          <t>Ronnie Stanley</t>
+          <t>Ezekiel Elliott</t>
         </is>
       </c>
       <c r="C54" s="16" t="inlineStr">
         <is>
-          <t>OT</t>
-        </is>
-      </c>
-      <c r="D54" s="17" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>RB</t>
+        </is>
+      </c>
+      <c r="D54" s="26" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E54" s="16" t="n">
@@ -3179,7 +3179,7 @@
       </c>
       <c r="H54" s="19" t="inlineStr">
         <is>
-          <t>Multiple All-Pro and Pro Bowl offensive tackle; cornerstone left tackle.</t>
+          <t>Multiple Pro Bowl and All-Pro running back with over 9,000 career rushing yards.</t>
         </is>
       </c>
     </row>
@@ -3189,12 +3189,12 @@
       </c>
       <c r="B55" s="21" t="inlineStr">
         <is>
-          <t>Ezekiel Elliott</t>
+          <t>Trey McBride</t>
         </is>
       </c>
       <c r="C55" s="22" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D55" s="23" t="inlineStr">
@@ -3203,7 +3203,7 @@
         </is>
       </c>
       <c r="E55" s="22" t="n">
-        <v>2016</v>
+        <v>2022</v>
       </c>
       <c r="F55" s="29" t="inlineStr">
         <is>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="H55" s="25" t="inlineStr">
         <is>
-          <t>Multiple Pro Bowl and All-Pro running back with over 9,000 career rushing yards.</t>
+          <t>Pro Bowl tight end and one of the league's most productive young receiving tight ends.</t>
         </is>
       </c>
     </row>
@@ -3227,12 +3227,12 @@
       </c>
       <c r="B56" s="15" t="inlineStr">
         <is>
-          <t>Trey McBride</t>
+          <t>Bijan Robinson</t>
         </is>
       </c>
       <c r="C56" s="16" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D56" s="26" t="inlineStr">
@@ -3241,7 +3241,7 @@
         </is>
       </c>
       <c r="E56" s="16" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="F56" s="28" t="inlineStr">
         <is>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="H56" s="19" t="inlineStr">
         <is>
-          <t>Pro Bowl tight end and one of the league's most productive young receiving tight ends.</t>
+          <t>Pro Bowl running back and one of the NFL's most productive young offensive players.</t>
         </is>
       </c>
     </row>
@@ -3265,12 +3265,12 @@
       </c>
       <c r="B57" s="21" t="inlineStr">
         <is>
-          <t>Bijan Robinson</t>
+          <t>Brock Bowers</t>
         </is>
       </c>
       <c r="C57" s="22" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D57" s="23" t="inlineStr">
@@ -3279,7 +3279,7 @@
         </is>
       </c>
       <c r="E57" s="22" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F57" s="29" t="inlineStr">
         <is>
@@ -3293,7 +3293,7 @@
       </c>
       <c r="H57" s="25" t="inlineStr">
         <is>
-          <t>Pro Bowl running back and one of the NFL's most productive young offensive players.</t>
+          <t>Pro Bowl tight end and one of the NFL's most productive young playmakers.</t>
         </is>
       </c>
     </row>
@@ -3303,25 +3303,25 @@
       </c>
       <c r="B58" s="15" t="inlineStr">
         <is>
-          <t>Brock Bowers</t>
+          <t>George Karlaftis III</t>
         </is>
       </c>
       <c r="C58" s="16" t="inlineStr">
         <is>
-          <t>TE</t>
-        </is>
-      </c>
-      <c r="D58" s="26" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>EDGE</t>
+        </is>
+      </c>
+      <c r="D58" s="17" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E58" s="16" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="F58" s="28" t="inlineStr">
         <is>
-          <t>75.5</t>
+          <t>75.0</t>
         </is>
       </c>
       <c r="G58" s="28" t="inlineStr">
@@ -3331,7 +3331,7 @@
       </c>
       <c r="H58" s="19" t="inlineStr">
         <is>
-          <t>Pro Bowl tight end and one of the NFL's most productive young playmakers.</t>
+          <t>Productive edge rusher and Super Bowl champion.</t>
         </is>
       </c>
     </row>
@@ -3341,25 +3341,25 @@
       </c>
       <c r="B59" s="21" t="inlineStr">
         <is>
-          <t>George Karlaftis III</t>
+          <t>Jaxon Smith-Njigba</t>
         </is>
       </c>
       <c r="C59" s="22" t="inlineStr">
         <is>
-          <t>EDGE</t>
-        </is>
-      </c>
-      <c r="D59" s="27" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>WR</t>
+        </is>
+      </c>
+      <c r="D59" s="23" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E59" s="22" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="F59" s="29" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>74.8</t>
         </is>
       </c>
       <c r="G59" s="29" t="inlineStr">
@@ -3369,7 +3369,7 @@
       </c>
       <c r="H59" s="25" t="inlineStr">
         <is>
-          <t>Productive edge rusher and Super Bowl champion.</t>
+          <t>Productive receiver and emerging focal point in the passing game. Super Bowl LX champion.</t>
         </is>
       </c>
     </row>
@@ -3379,25 +3379,25 @@
       </c>
       <c r="B60" s="15" t="inlineStr">
         <is>
-          <t>Jaxon Smith-Njigba</t>
+          <t>Jared Verse</t>
         </is>
       </c>
       <c r="C60" s="16" t="inlineStr">
         <is>
-          <t>WR</t>
-        </is>
-      </c>
-      <c r="D60" s="26" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>EDGE</t>
+        </is>
+      </c>
+      <c r="D60" s="17" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E60" s="16" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F60" s="28" t="inlineStr">
         <is>
-          <t>74.8</t>
+          <t>74.6</t>
         </is>
       </c>
       <c r="G60" s="28" t="inlineStr">
@@ -3407,7 +3407,7 @@
       </c>
       <c r="H60" s="19" t="inlineStr">
         <is>
-          <t>Productive receiver and emerging focal point in the passing game. Super Bowl LX champion.</t>
+          <t>DROY winner and impact pass rusher; cornerstone defensive player.</t>
         </is>
       </c>
     </row>
@@ -3417,17 +3417,17 @@
       </c>
       <c r="B61" s="21" t="inlineStr">
         <is>
-          <t>Jared Verse</t>
+          <t>Jayden Daniels</t>
         </is>
       </c>
       <c r="C61" s="22" t="inlineStr">
         <is>
-          <t>EDGE</t>
-        </is>
-      </c>
-      <c r="D61" s="27" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>QB</t>
+        </is>
+      </c>
+      <c r="D61" s="23" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E61" s="22" t="n">
@@ -3445,7 +3445,7 @@
       </c>
       <c r="H61" s="25" t="inlineStr">
         <is>
-          <t>DROY winner and impact pass rusher; cornerstone defensive player.</t>
+          <t>Pro Bowl quarterback who emerged as one of the league's top young passers.</t>
         </is>
       </c>
     </row>
@@ -3455,25 +3455,25 @@
       </c>
       <c r="B62" s="15" t="inlineStr">
         <is>
-          <t>Jayden Daniels</t>
+          <t>Melvin Gordon</t>
         </is>
       </c>
       <c r="C62" s="16" t="inlineStr">
         <is>
-          <t>QB</t>
-        </is>
-      </c>
-      <c r="D62" s="26" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>RB</t>
+        </is>
+      </c>
+      <c r="D62" s="17" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E62" s="16" t="n">
-        <v>2024</v>
+        <v>2015</v>
       </c>
       <c r="F62" s="28" t="inlineStr">
         <is>
-          <t>74.6</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="G62" s="28" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="H62" s="19" t="inlineStr">
         <is>
-          <t>Pro Bowl quarterback who emerged as one of the league's top young passers.</t>
+          <t>Multiple Pro Bowl running back with over 6,000 career rushing yards.</t>
         </is>
       </c>
     </row>
@@ -3977,7 +3977,7 @@
       </c>
       <c r="H75" s="25" t="inlineStr">
         <is>
-          <t>All-Pro linebacker and key defensive contributor; Super Bowl champion.</t>
+          <t>All-Pro linebacker and key defensive contributor.</t>
         </is>
       </c>
     </row>
@@ -5003,7 +5003,7 @@
       </c>
       <c r="H102" s="19" t="inlineStr">
         <is>
-          <t>Pro Bowl receiver and key contributor on a Super Bowl championship team; Super Bowl champion.</t>
+          <t>Pro Bowl receiver and key contributor on a Super Bowl championship team.</t>
         </is>
       </c>
     </row>
@@ -5155,7 +5155,7 @@
       </c>
       <c r="H106" s="19" t="inlineStr">
         <is>
-          <t>Defensive tackle and key contributor on championship-caliber defenses; Super Bowl champion.</t>
+          <t>Defensive tackle and key contributor on championship-caliber defenses.</t>
         </is>
       </c>
     </row>
@@ -5193,7 +5193,7 @@
       </c>
       <c r="H107" s="25" t="inlineStr">
         <is>
-          <t>Edge defender and key contributor on playoff defenses; Super Bowl champion.</t>
+          <t>Edge defender and key contributor on playoff defenses.</t>
         </is>
       </c>
     </row>
@@ -5801,7 +5801,7 @@
       </c>
       <c r="H123" s="25" t="inlineStr">
         <is>
-          <t>Pro Bowl quarterback who played a major role in a Super Bowl-winning season; Super Bowl champion.</t>
+          <t>Pro Bowl quarterback who played a major role in a Super Bowl-winning season.</t>
         </is>
       </c>
     </row>
@@ -5915,7 +5915,7 @@
       </c>
       <c r="H126" s="19" t="inlineStr">
         <is>
-          <t>Rotational edge rusher who contributed across multiple teams; Super Bowl champion.</t>
+          <t>Rotational edge rusher who contributed across multiple teams.</t>
         </is>
       </c>
     </row>
@@ -7093,7 +7093,7 @@
       </c>
       <c r="H157" s="25" t="inlineStr">
         <is>
-          <t>Starting offensive lineman whose career has been impacted by injuries; Super Bowl champion.</t>
+          <t>Starting offensive lineman whose career has been impacted by injuries.</t>
         </is>
       </c>
     </row>
@@ -7359,7 +7359,7 @@
       </c>
       <c r="H164" s="19" t="inlineStr">
         <is>
-          <t>Linebacker whose career has been impacted by injuries; Super Bowl champion.</t>
+          <t>Linebacker whose career has been impacted by injuries.</t>
         </is>
       </c>
     </row>
@@ -7369,12 +7369,12 @@
       </c>
       <c r="B165" s="21" t="inlineStr">
         <is>
-          <t>Cameron Erving</t>
+          <t>Jaylon Smith</t>
         </is>
       </c>
       <c r="C165" s="22" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>OLB</t>
         </is>
       </c>
       <c r="D165" s="27" t="inlineStr">
@@ -7383,11 +7383,11 @@
         </is>
       </c>
       <c r="E165" s="22" t="n">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="F165" s="20" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="G165" s="20" t="inlineStr">
@@ -7397,7 +7397,7 @@
       </c>
       <c r="H165" s="25" t="inlineStr">
         <is>
-          <t>Versatile offensive lineman with extensive starting experience; 2x Super Bowl champion. [PFR correction — SB Win 1→2.]</t>
+          <t>Pro Bowl linebacker who overcame a significant college injury to become a productive starter.</t>
         </is>
       </c>
     </row>
@@ -7407,12 +7407,12 @@
       </c>
       <c r="B166" s="15" t="inlineStr">
         <is>
-          <t>Cam Akers</t>
+          <t>Chukwuma Okorafor</t>
         </is>
       </c>
       <c r="C166" s="16" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>OT</t>
         </is>
       </c>
       <c r="D166" s="17" t="inlineStr">
@@ -7421,11 +7421,11 @@
         </is>
       </c>
       <c r="E166" s="16" t="n">
-        <v>2020</v>
+        <v>2018</v>
       </c>
       <c r="F166" s="14" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="G166" s="14" t="inlineStr">
@@ -7435,7 +7435,7 @@
       </c>
       <c r="H166" s="19" t="inlineStr">
         <is>
-          <t>Running back who returned from a major injury and contributed on multiple teams; 2x Super Bowl champion.</t>
+          <t>Long-term NFL starting offensive tackle.</t>
         </is>
       </c>
     </row>
@@ -7445,12 +7445,12 @@
       </c>
       <c r="B167" s="21" t="inlineStr">
         <is>
-          <t>Jaylon Smith</t>
+          <t>Grant Delpit</t>
         </is>
       </c>
       <c r="C167" s="22" t="inlineStr">
         <is>
-          <t>OLB</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D167" s="27" t="inlineStr">
@@ -7459,7 +7459,7 @@
         </is>
       </c>
       <c r="E167" s="22" t="n">
-        <v>2016</v>
+        <v>2020</v>
       </c>
       <c r="F167" s="20" t="inlineStr">
         <is>
@@ -7473,7 +7473,7 @@
       </c>
       <c r="H167" s="25" t="inlineStr">
         <is>
-          <t>Pro Bowl linebacker who overcame a significant college injury to become a productive starter.</t>
+          <t>Starting safety and productive defensive contributor.</t>
         </is>
       </c>
     </row>
@@ -7483,21 +7483,21 @@
       </c>
       <c r="B168" s="15" t="inlineStr">
         <is>
-          <t>Chukwuma Okorafor</t>
+          <t>Zack Moss</t>
         </is>
       </c>
       <c r="C168" s="16" t="inlineStr">
         <is>
-          <t>OT</t>
-        </is>
-      </c>
-      <c r="D168" s="17" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>RB</t>
+        </is>
+      </c>
+      <c r="D168" s="26" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E168" s="16" t="n">
-        <v>2018</v>
+        <v>2020</v>
       </c>
       <c r="F168" s="14" t="inlineStr">
         <is>
@@ -7511,7 +7511,7 @@
       </c>
       <c r="H168" s="19" t="inlineStr">
         <is>
-          <t>Long-term NFL starting offensive tackle.</t>
+          <t>Running back with multiple productive rushing seasons.</t>
         </is>
       </c>
     </row>
@@ -7521,12 +7521,12 @@
       </c>
       <c r="B169" s="21" t="inlineStr">
         <is>
-          <t>Grant Delpit</t>
+          <t>Cameron Erving</t>
         </is>
       </c>
       <c r="C169" s="22" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D169" s="27" t="inlineStr">
@@ -7535,11 +7535,11 @@
         </is>
       </c>
       <c r="E169" s="22" t="n">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="F169" s="20" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>55.5</t>
         </is>
       </c>
       <c r="G169" s="20" t="inlineStr">
@@ -7549,7 +7549,7 @@
       </c>
       <c r="H169" s="25" t="inlineStr">
         <is>
-          <t>Starting safety and productive defensive contributor.</t>
+          <t>Versatile offensive lineman with extensive starting experience.</t>
         </is>
       </c>
     </row>
@@ -7559,12 +7559,12 @@
       </c>
       <c r="B170" s="15" t="inlineStr">
         <is>
-          <t>Zack Moss</t>
+          <t>Kyle Fuller</t>
         </is>
       </c>
       <c r="C170" s="16" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D170" s="26" t="inlineStr">
@@ -7573,11 +7573,11 @@
         </is>
       </c>
       <c r="E170" s="16" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="F170" s="14" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>55.5</t>
         </is>
       </c>
       <c r="G170" s="14" t="inlineStr">
@@ -7587,7 +7587,7 @@
       </c>
       <c r="H170" s="19" t="inlineStr">
         <is>
-          <t>Running back with multiple productive rushing seasons.</t>
+          <t>Multiple Pro Bowl and All-Pro cornerback known for creating turnovers.</t>
         </is>
       </c>
     </row>
@@ -7597,21 +7597,21 @@
       </c>
       <c r="B171" s="21" t="inlineStr">
         <is>
-          <t>Kyle Fuller</t>
+          <t>Cam Akers</t>
         </is>
       </c>
       <c r="C171" s="22" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D171" s="23" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>RB</t>
+        </is>
+      </c>
+      <c r="D171" s="27" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E171" s="22" t="n">
-        <v>2017</v>
+        <v>2020</v>
       </c>
       <c r="F171" s="20" t="inlineStr">
         <is>
@@ -7625,7 +7625,7 @@
       </c>
       <c r="H171" s="25" t="inlineStr">
         <is>
-          <t>Multiple Pro Bowl and All-Pro cornerback known for creating turnovers.</t>
+          <t>Running back who returned from a major injury and contributed on multiple teams.; Super Bowl champion (2nd ring was practice squad — not a roster ring). [PFR correction — SB Win 2→1.]</t>
         </is>
       </c>
     </row>
@@ -7635,25 +7635,25 @@
       </c>
       <c r="B172" s="15" t="inlineStr">
         <is>
-          <t>Caden Sterns</t>
+          <t>Deon Bush</t>
         </is>
       </c>
       <c r="C172" s="16" t="inlineStr">
         <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="D172" s="26" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>SS</t>
+        </is>
+      </c>
+      <c r="D172" s="17" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E172" s="16" t="n">
-        <v>2021</v>
+        <v>2016</v>
       </c>
       <c r="F172" s="14" t="inlineStr">
         <is>
-          <t>55.5</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G172" s="14" t="inlineStr">
@@ -7663,7 +7663,7 @@
       </c>
       <c r="H172" s="19" t="inlineStr">
         <is>
-          <t>Safety whose career has been impacted by injuries; Super Bowl champion. [PFR correction — SB Win 0→1.]</t>
+          <t>Super Bowl champion safety and long-term depth contributor.</t>
         </is>
       </c>
     </row>
@@ -7673,12 +7673,12 @@
       </c>
       <c r="B173" s="21" t="inlineStr">
         <is>
-          <t>Christian Haynes</t>
+          <t>Jesse James</t>
         </is>
       </c>
       <c r="C173" s="22" t="inlineStr">
         <is>
-          <t>OL</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D173" s="27" t="inlineStr">
@@ -7687,11 +7687,11 @@
         </is>
       </c>
       <c r="E173" s="22" t="n">
-        <v>2024</v>
+        <v>2015</v>
       </c>
       <c r="F173" s="20" t="inlineStr">
         <is>
-          <t>55.5</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="G173" s="20" t="inlineStr">
@@ -7701,7 +7701,7 @@
       </c>
       <c r="H173" s="25" t="inlineStr">
         <is>
-          <t>Interior offensive lineman with starting potential and early NFL experience; Super Bowl champion. [PFR correction — SB Win 0→1.]</t>
+          <t>Long-term NFL tight end and reliable red-zone contributor.</t>
         </is>
       </c>
     </row>
@@ -7711,12 +7711,12 @@
       </c>
       <c r="B174" s="15" t="inlineStr">
         <is>
-          <t>Deon Bush</t>
+          <t>Trae Waynes</t>
         </is>
       </c>
       <c r="C174" s="16" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D174" s="17" t="inlineStr">
@@ -7725,11 +7725,11 @@
         </is>
       </c>
       <c r="E174" s="16" t="n">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="F174" s="14" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="G174" s="14" t="inlineStr">
@@ -7739,7 +7739,7 @@
       </c>
       <c r="H174" s="19" t="inlineStr">
         <is>
-          <t>Super Bowl champion safety and long-term depth contributor.</t>
+          <t>Starting cornerback whose career was impacted by injuries.</t>
         </is>
       </c>
     </row>
@@ -7749,7 +7749,7 @@
       </c>
       <c r="B175" s="21" t="inlineStr">
         <is>
-          <t>Jesse James</t>
+          <t>Nick Vannett</t>
         </is>
       </c>
       <c r="C175" s="22" t="inlineStr">
@@ -7757,13 +7757,13 @@
           <t>TE</t>
         </is>
       </c>
-      <c r="D175" s="27" t="inlineStr">
-        <is>
-          <t>Matt</t>
+      <c r="D175" s="23" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E175" s="22" t="n">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="F175" s="20" t="inlineStr">
         <is>
@@ -7777,7 +7777,7 @@
       </c>
       <c r="H175" s="25" t="inlineStr">
         <is>
-          <t>Long-term NFL tight end and reliable red-zone contributor.</t>
+          <t>Blocking tight end and reliable depth contributor.</t>
         </is>
       </c>
     </row>
@@ -7787,7 +7787,7 @@
       </c>
       <c r="B176" s="15" t="inlineStr">
         <is>
-          <t>Trae Waynes</t>
+          <t>Artie Burns</t>
         </is>
       </c>
       <c r="C176" s="16" t="inlineStr">
@@ -7795,13 +7795,13 @@
           <t>CB</t>
         </is>
       </c>
-      <c r="D176" s="17" t="inlineStr">
-        <is>
-          <t>Matt</t>
+      <c r="D176" s="26" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E176" s="16" t="n">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="F176" s="14" t="inlineStr">
         <is>
@@ -7815,7 +7815,7 @@
       </c>
       <c r="H176" s="19" t="inlineStr">
         <is>
-          <t>Starting cornerback whose career was impacted by injuries.</t>
+          <t>Cornerback who contributed as a starter and depth player during his NFL career.</t>
         </is>
       </c>
     </row>
@@ -7825,21 +7825,21 @@
       </c>
       <c r="B177" s="21" t="inlineStr">
         <is>
-          <t>Nick Vannett</t>
+          <t>Mitchell Trubisky</t>
         </is>
       </c>
       <c r="C177" s="22" t="inlineStr">
         <is>
-          <t>TE</t>
-        </is>
-      </c>
-      <c r="D177" s="23" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>QB</t>
+        </is>
+      </c>
+      <c r="D177" s="27" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E177" s="22" t="n">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="F177" s="20" t="inlineStr">
         <is>
@@ -7853,7 +7853,7 @@
       </c>
       <c r="H177" s="25" t="inlineStr">
         <is>
-          <t>Blocking tight end and reliable depth contributor.</t>
+          <t>Pro Bowl quarterback who started multiple seasons and led the Bears to a playoff appearance.</t>
         </is>
       </c>
     </row>
@@ -7863,21 +7863,21 @@
       </c>
       <c r="B178" s="15" t="inlineStr">
         <is>
-          <t>Artie Burns</t>
+          <t>Michael Gallup</t>
         </is>
       </c>
       <c r="C178" s="16" t="inlineStr">
         <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="D178" s="26" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>WR</t>
+        </is>
+      </c>
+      <c r="D178" s="17" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E178" s="16" t="n">
-        <v>2016</v>
+        <v>2018</v>
       </c>
       <c r="F178" s="14" t="inlineStr">
         <is>
@@ -7891,7 +7891,7 @@
       </c>
       <c r="H178" s="19" t="inlineStr">
         <is>
-          <t>Cornerback who contributed as a starter and depth player during his NFL career.</t>
+          <t>Productive starting receiver with multiple 800+ yard seasons.</t>
         </is>
       </c>
     </row>
@@ -7901,12 +7901,12 @@
       </c>
       <c r="B179" s="21" t="inlineStr">
         <is>
-          <t>Mitchell Trubisky</t>
+          <t>Maurice Hurst Jr.</t>
         </is>
       </c>
       <c r="C179" s="22" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="D179" s="27" t="inlineStr">
@@ -7915,7 +7915,7 @@
         </is>
       </c>
       <c r="E179" s="22" t="n">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="F179" s="20" t="inlineStr">
         <is>
@@ -7929,7 +7929,7 @@
       </c>
       <c r="H179" s="25" t="inlineStr">
         <is>
-          <t>Pro Bowl quarterback who started multiple seasons and led the Bears to a playoff appearance.</t>
+          <t>Defensive tackle who contributed as a rotational starter and depth player.</t>
         </is>
       </c>
     </row>
@@ -7939,21 +7939,21 @@
       </c>
       <c r="B180" s="15" t="inlineStr">
         <is>
-          <t>Michael Gallup</t>
+          <t>Teven Jenkins</t>
         </is>
       </c>
       <c r="C180" s="16" t="inlineStr">
         <is>
-          <t>WR</t>
-        </is>
-      </c>
-      <c r="D180" s="17" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>OL</t>
+        </is>
+      </c>
+      <c r="D180" s="26" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E180" s="16" t="n">
-        <v>2018</v>
+        <v>2021</v>
       </c>
       <c r="F180" s="14" t="inlineStr">
         <is>
@@ -7967,7 +7967,7 @@
       </c>
       <c r="H180" s="19" t="inlineStr">
         <is>
-          <t>Productive starting receiver with multiple 800+ yard seasons.</t>
+          <t>Starting offensive lineman known for versatility and physical play.</t>
         </is>
       </c>
     </row>
@@ -7977,21 +7977,21 @@
       </c>
       <c r="B181" s="21" t="inlineStr">
         <is>
-          <t>Maurice Hurst Jr.</t>
+          <t>Malcolm Koonce</t>
         </is>
       </c>
       <c r="C181" s="22" t="inlineStr">
         <is>
-          <t>DT</t>
-        </is>
-      </c>
-      <c r="D181" s="27" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>EDGE</t>
+        </is>
+      </c>
+      <c r="D181" s="23" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E181" s="22" t="n">
-        <v>2018</v>
+        <v>2021</v>
       </c>
       <c r="F181" s="20" t="inlineStr">
         <is>
@@ -8005,7 +8005,7 @@
       </c>
       <c r="H181" s="25" t="inlineStr">
         <is>
-          <t>Defensive tackle who contributed as a rotational starter and depth player.</t>
+          <t>Edge rusher who developed into a productive defensive contributor.</t>
         </is>
       </c>
     </row>
@@ -8015,12 +8015,12 @@
       </c>
       <c r="B182" s="15" t="inlineStr">
         <is>
-          <t>Teven Jenkins</t>
+          <t>Zaven Collins</t>
         </is>
       </c>
       <c r="C182" s="16" t="inlineStr">
         <is>
-          <t>OL</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D182" s="26" t="inlineStr">
@@ -8043,7 +8043,7 @@
       </c>
       <c r="H182" s="19" t="inlineStr">
         <is>
-          <t>Starting offensive lineman known for versatility and physical play.</t>
+          <t>Linebacker and defensive contributor with starting experience.</t>
         </is>
       </c>
     </row>
@@ -8053,12 +8053,12 @@
       </c>
       <c r="B183" s="21" t="inlineStr">
         <is>
-          <t>Malcolm Koonce</t>
+          <t>Isaiah Mcduffie</t>
         </is>
       </c>
       <c r="C183" s="22" t="inlineStr">
         <is>
-          <t>EDGE</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D183" s="23" t="inlineStr">
@@ -8081,7 +8081,7 @@
       </c>
       <c r="H183" s="25" t="inlineStr">
         <is>
-          <t>Edge rusher who developed into a productive defensive contributor.</t>
+          <t>Linebacker and special teams contributor who earned a larger defensive role.</t>
         </is>
       </c>
     </row>
@@ -8091,12 +8091,12 @@
       </c>
       <c r="B184" s="15" t="inlineStr">
         <is>
-          <t>Zaven Collins</t>
+          <t>Caden Sterns</t>
         </is>
       </c>
       <c r="C184" s="16" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D184" s="26" t="inlineStr">
@@ -8119,7 +8119,7 @@
       </c>
       <c r="H184" s="19" t="inlineStr">
         <is>
-          <t>Linebacker and defensive contributor with starting experience.</t>
+          <t>Safety whose career has been impacted by injuries.</t>
         </is>
       </c>
     </row>
@@ -8129,21 +8129,21 @@
       </c>
       <c r="B185" s="21" t="inlineStr">
         <is>
-          <t>Isaiah Mcduffie</t>
+          <t>Chig Okonkwo</t>
         </is>
       </c>
       <c r="C185" s="22" t="inlineStr">
         <is>
-          <t>LB</t>
-        </is>
-      </c>
-      <c r="D185" s="23" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>TE</t>
+        </is>
+      </c>
+      <c r="D185" s="27" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E185" s="22" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="F185" s="20" t="inlineStr">
         <is>
@@ -8157,7 +8157,7 @@
       </c>
       <c r="H185" s="25" t="inlineStr">
         <is>
-          <t>Linebacker and special teams contributor who earned a larger defensive role.</t>
+          <t>Athletic tight end and productive receiving contributor.</t>
         </is>
       </c>
     </row>
@@ -8167,12 +8167,12 @@
       </c>
       <c r="B186" s="15" t="inlineStr">
         <is>
-          <t>Chig Okonkwo</t>
+          <t>Daxton Hill</t>
         </is>
       </c>
       <c r="C186" s="16" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D186" s="17" t="inlineStr">
@@ -8195,7 +8195,7 @@
       </c>
       <c r="H186" s="19" t="inlineStr">
         <is>
-          <t>Athletic tight end and productive receiving contributor.</t>
+          <t>Defensive back with starting experience in the secondary.</t>
         </is>
       </c>
     </row>
@@ -8205,12 +8205,12 @@
       </c>
       <c r="B187" s="21" t="inlineStr">
         <is>
-          <t>Daxton Hill</t>
+          <t>Darnell Washington</t>
         </is>
       </c>
       <c r="C187" s="22" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D187" s="27" t="inlineStr">
@@ -8219,7 +8219,7 @@
         </is>
       </c>
       <c r="E187" s="22" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="F187" s="20" t="inlineStr">
         <is>
@@ -8233,7 +8233,7 @@
       </c>
       <c r="H187" s="25" t="inlineStr">
         <is>
-          <t>Defensive back with starting experience in the secondary.</t>
+          <t>Blocking tight end known for versatility and physical play.</t>
         </is>
       </c>
     </row>
@@ -8243,12 +8243,12 @@
       </c>
       <c r="B188" s="15" t="inlineStr">
         <is>
-          <t>Darnell Washington</t>
+          <t>Sidy Sow</t>
         </is>
       </c>
       <c r="C188" s="16" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>OL</t>
         </is>
       </c>
       <c r="D188" s="17" t="inlineStr">
@@ -8271,7 +8271,7 @@
       </c>
       <c r="H188" s="19" t="inlineStr">
         <is>
-          <t>Blocking tight end known for versatility and physical play.</t>
+          <t>Offensive lineman with starting experience and positional versatility.</t>
         </is>
       </c>
     </row>
@@ -8281,12 +8281,12 @@
       </c>
       <c r="B189" s="21" t="inlineStr">
         <is>
-          <t>Sidy Sow</t>
+          <t>BJ Ojulari</t>
         </is>
       </c>
       <c r="C189" s="22" t="inlineStr">
         <is>
-          <t>OL</t>
+          <t>EDGE</t>
         </is>
       </c>
       <c r="D189" s="27" t="inlineStr">
@@ -8309,7 +8309,7 @@
       </c>
       <c r="H189" s="25" t="inlineStr">
         <is>
-          <t>Offensive lineman with starting experience and positional versatility.</t>
+          <t>Edge defender whose early career has been impacted by injury.</t>
         </is>
       </c>
     </row>
@@ -8319,12 +8319,12 @@
       </c>
       <c r="B190" s="15" t="inlineStr">
         <is>
-          <t>BJ Ojulari</t>
+          <t>Mazi Smith</t>
         </is>
       </c>
       <c r="C190" s="16" t="inlineStr">
         <is>
-          <t>EDGE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D190" s="17" t="inlineStr">
@@ -8347,7 +8347,7 @@
       </c>
       <c r="H190" s="19" t="inlineStr">
         <is>
-          <t>Edge defender whose early career has been impacted by injury.</t>
+          <t>Defensive tackle and contributor on the defensive front.</t>
         </is>
       </c>
     </row>
@@ -8357,17 +8357,17 @@
       </c>
       <c r="B191" s="21" t="inlineStr">
         <is>
-          <t>Mazi Smith</t>
+          <t>Henry To'oTo'o</t>
         </is>
       </c>
       <c r="C191" s="22" t="inlineStr">
         <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D191" s="27" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="D191" s="23" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E191" s="22" t="n">
@@ -8385,7 +8385,7 @@
       </c>
       <c r="H191" s="25" t="inlineStr">
         <is>
-          <t>Defensive tackle and contributor on the defensive front.</t>
+          <t>Starting linebacker and productive defensive contributor.</t>
         </is>
       </c>
     </row>
@@ -8395,21 +8395,21 @@
       </c>
       <c r="B192" s="15" t="inlineStr">
         <is>
-          <t>Henry To'oTo'o</t>
+          <t>Theo Johnson</t>
         </is>
       </c>
       <c r="C192" s="16" t="inlineStr">
         <is>
-          <t>LB</t>
-        </is>
-      </c>
-      <c r="D192" s="26" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>TE</t>
+        </is>
+      </c>
+      <c r="D192" s="17" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E192" s="16" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F192" s="14" t="inlineStr">
         <is>
@@ -8423,7 +8423,7 @@
       </c>
       <c r="H192" s="19" t="inlineStr">
         <is>
-          <t>Starting linebacker and productive defensive contributor.</t>
+          <t>Athletic tight end and developing receiving target.</t>
         </is>
       </c>
     </row>
@@ -8433,12 +8433,12 @@
       </c>
       <c r="B193" s="21" t="inlineStr">
         <is>
-          <t>Theo Johnson</t>
+          <t>Christian Haynes</t>
         </is>
       </c>
       <c r="C193" s="22" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>OL</t>
         </is>
       </c>
       <c r="D193" s="27" t="inlineStr">
@@ -8461,7 +8461,7 @@
       </c>
       <c r="H193" s="25" t="inlineStr">
         <is>
-          <t>Athletic tight end and developing receiving target.</t>
+          <t>Interior offensive lineman with starting potential and early NFL experience.</t>
         </is>
       </c>
     </row>
@@ -9867,7 +9867,7 @@
       </c>
       <c r="H230" s="19" t="inlineStr">
         <is>
-          <t>Edge defender and rotational contributor on championship-caliber teams; Super Bowl champion.</t>
+          <t>Edge defender and rotational contributor on championship-caliber teams.</t>
         </is>
       </c>
     </row>
@@ -9905,7 +9905,7 @@
       </c>
       <c r="H231" s="25" t="inlineStr">
         <is>
-          <t>Cornerback who contributed on defense and special teams; Super Bowl champion.</t>
+          <t>Cornerback who contributed on defense and special teams.</t>
         </is>
       </c>
     </row>
@@ -9943,7 +9943,7 @@
       </c>
       <c r="H232" s="19" t="inlineStr">
         <is>
-          <t>Linebacker who contributed on defense and special teams; Super Bowl champion.</t>
+          <t>Linebacker who contributed on defense and special teams.</t>
         </is>
       </c>
     </row>
@@ -11035,7 +11035,7 @@
       </c>
       <c r="F261" s="22" t="inlineStr">
         <is>
-          <t>44.6</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="G261" s="22" t="inlineStr">
@@ -11045,7 +11045,7 @@
       </c>
       <c r="H261" s="25" t="inlineStr">
         <is>
-          <t>OROY winner whose promising career was significantly impacted by injuries. [PFR correction — OROY 0→1.]</t>
+          <t>OROY winner whose promising career was significantly impacted by injuries.</t>
         </is>
       </c>
     </row>
@@ -11187,7 +11187,7 @@
       </c>
       <c r="F265" s="22" t="inlineStr">
         <is>
-          <t>43.5</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G265" s="22" t="inlineStr">
@@ -11197,7 +11197,7 @@
       </c>
       <c r="H265" s="25" t="inlineStr">
         <is>
-          <t>Long-term NFL backup quarterback who spent over a decade in the league as a reserve and spot starter; Super Bowl champion. [PFR correction — SB Win 0→1.]</t>
+          <t>Long-term NFL backup quarterback who spent over a decade in the league as a reserve and spot starter.</t>
         </is>
       </c>
     </row>
@@ -11891,12 +11891,12 @@
       </c>
       <c r="B284" s="15" t="inlineStr">
         <is>
-          <t>Corey Coleman</t>
+          <t>Chase Young</t>
         </is>
       </c>
       <c r="C284" s="16" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>EDGE</t>
         </is>
       </c>
       <c r="D284" s="26" t="inlineStr">
@@ -11905,11 +11905,11 @@
         </is>
       </c>
       <c r="E284" s="16" t="n">
-        <v>2016</v>
+        <v>2020</v>
       </c>
       <c r="F284" s="26" t="inlineStr">
         <is>
-          <t>35.5</t>
+          <t>34.6</t>
         </is>
       </c>
       <c r="G284" s="26" t="inlineStr">
@@ -11919,7 +11919,7 @@
       </c>
       <c r="H284" s="19" t="inlineStr">
         <is>
-          <t>Receiver whose NFL career was limited by injuries and inconsistency; Super Bowl champion. [PFR correction — SB Win 0→1.]</t>
+          <t>DROY winner and Pro Bowl edge rusher.</t>
         </is>
       </c>
     </row>
@@ -11929,25 +11929,25 @@
       </c>
       <c r="B285" s="21" t="inlineStr">
         <is>
-          <t>Chase Young</t>
+          <t>Taiwan Jones</t>
         </is>
       </c>
       <c r="C285" s="22" t="inlineStr">
         <is>
-          <t>EDGE</t>
-        </is>
-      </c>
-      <c r="D285" s="23" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>ILB</t>
+        </is>
+      </c>
+      <c r="D285" s="27" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E285" s="22" t="n">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="F285" s="23" t="inlineStr">
         <is>
-          <t>34.6</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="G285" s="23" t="inlineStr">
@@ -11957,7 +11957,7 @@
       </c>
       <c r="H285" s="25" t="inlineStr">
         <is>
-          <t>DROY winner and Pro Bowl edge rusher.</t>
+          <t>Special teams contributor and depth running back with a lengthy NFL career.</t>
         </is>
       </c>
     </row>
@@ -11967,12 +11967,12 @@
       </c>
       <c r="B286" s="15" t="inlineStr">
         <is>
-          <t>Taiwan Jones</t>
+          <t>Laquon Treadwell</t>
         </is>
       </c>
       <c r="C286" s="16" t="inlineStr">
         <is>
-          <t>ILB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D286" s="17" t="inlineStr">
@@ -11981,7 +11981,7 @@
         </is>
       </c>
       <c r="E286" s="16" t="n">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="F286" s="26" t="inlineStr">
         <is>
@@ -11995,7 +11995,7 @@
       </c>
       <c r="H286" s="19" t="inlineStr">
         <is>
-          <t>Special teams contributor and depth running back with a lengthy NFL career.</t>
+          <t>Receiver who contributed in reserve roles across multiple teams.</t>
         </is>
       </c>
     </row>
@@ -12005,7 +12005,7 @@
       </c>
       <c r="B287" s="21" t="inlineStr">
         <is>
-          <t>Laquon Treadwell</t>
+          <t>Corey Coleman</t>
         </is>
       </c>
       <c r="C287" s="22" t="inlineStr">
@@ -12013,9 +12013,9 @@
           <t>WR</t>
         </is>
       </c>
-      <c r="D287" s="27" t="inlineStr">
-        <is>
-          <t>Matt</t>
+      <c r="D287" s="23" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E287" s="22" t="n">
@@ -12033,7 +12033,7 @@
       </c>
       <c r="H287" s="25" t="inlineStr">
         <is>
-          <t>Receiver who contributed in reserve roles across multiple teams.</t>
+          <t>Receiver whose NFL career was limited by injuries and inconsistency.</t>
         </is>
       </c>
     </row>
@@ -12081,25 +12081,25 @@
       </c>
       <c r="B289" s="21" t="inlineStr">
         <is>
-          <t>Obi Melifonwu</t>
+          <t>Matt Barkley</t>
         </is>
       </c>
       <c r="C289" s="22" t="inlineStr">
         <is>
-          <t>SS</t>
-        </is>
-      </c>
-      <c r="D289" s="27" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>QB</t>
+        </is>
+      </c>
+      <c r="D289" s="23" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E289" s="22" t="n">
-        <v>2017</v>
+        <v>2013</v>
       </c>
       <c r="F289" s="23" t="inlineStr">
         <is>
-          <t>33.5</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="G289" s="23" t="inlineStr">
@@ -12109,7 +12109,7 @@
       </c>
       <c r="H289" s="25" t="inlineStr">
         <is>
-          <t>Defensive back whose NFL career was limited by injuries; Super Bowl champion. [PFR correction — SB Win 0→1.]</t>
+          <t>Career backup quarterback who provided depth across multiple organizations.</t>
         </is>
       </c>
     </row>
@@ -12119,12 +12119,12 @@
       </c>
       <c r="B290" s="15" t="inlineStr">
         <is>
-          <t>Deandre Baker</t>
+          <t>Robert Nkemdiche</t>
         </is>
       </c>
       <c r="C290" s="16" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="D290" s="17" t="inlineStr">
@@ -12133,11 +12133,11 @@
         </is>
       </c>
       <c r="E290" s="16" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="F290" s="26" t="inlineStr">
         <is>
-          <t>33.5</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="G290" s="26" t="inlineStr">
@@ -12147,7 +12147,7 @@
       </c>
       <c r="H290" s="19" t="inlineStr">
         <is>
-          <t>Cornerback whose NFL career was limited by injuries and availability issues; Super Bowl champion. [PFR correction — SB Win 0→1.]</t>
+          <t>Defensive lineman whose NFL career did not meet first-round expectations.</t>
         </is>
       </c>
     </row>
@@ -12157,21 +12157,21 @@
       </c>
       <c r="B291" s="21" t="inlineStr">
         <is>
-          <t>Matt Barkley</t>
+          <t>Kevin Dodd</t>
         </is>
       </c>
       <c r="C291" s="22" t="inlineStr">
         <is>
-          <t>QB</t>
-        </is>
-      </c>
-      <c r="D291" s="23" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D291" s="27" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E291" s="22" t="n">
-        <v>2013</v>
+        <v>2016</v>
       </c>
       <c r="F291" s="23" t="inlineStr">
         <is>
@@ -12185,7 +12185,7 @@
       </c>
       <c r="H291" s="25" t="inlineStr">
         <is>
-          <t>Career backup quarterback who provided depth across multiple organizations.</t>
+          <t>Edge rusher whose NFL career was limited by injuries.</t>
         </is>
       </c>
     </row>
@@ -12195,12 +12195,12 @@
       </c>
       <c r="B292" s="15" t="inlineStr">
         <is>
-          <t>Robert Nkemdiche</t>
+          <t>Scooby Wright III</t>
         </is>
       </c>
       <c r="C292" s="16" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>ILB</t>
         </is>
       </c>
       <c r="D292" s="17" t="inlineStr">
@@ -12223,7 +12223,7 @@
       </c>
       <c r="H292" s="19" t="inlineStr">
         <is>
-          <t>Defensive lineman whose NFL career did not meet first-round expectations.</t>
+          <t>Linebacker and special teams contributor during his professional career.</t>
         </is>
       </c>
     </row>
@@ -12233,17 +12233,17 @@
       </c>
       <c r="B293" s="21" t="inlineStr">
         <is>
-          <t>Kevin Dodd</t>
+          <t>Vadal Alexander</t>
         </is>
       </c>
       <c r="C293" s="22" t="inlineStr">
         <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D293" s="27" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>OG</t>
+        </is>
+      </c>
+      <c r="D293" s="23" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E293" s="22" t="n">
@@ -12261,7 +12261,7 @@
       </c>
       <c r="H293" s="25" t="inlineStr">
         <is>
-          <t>Edge rusher whose NFL career was limited by injuries.</t>
+          <t>Offensive lineman who provided depth during his NFL career.</t>
         </is>
       </c>
     </row>
@@ -12271,17 +12271,17 @@
       </c>
       <c r="B294" s="15" t="inlineStr">
         <is>
-          <t>Scooby Wright III</t>
+          <t>Jeremy Cash</t>
         </is>
       </c>
       <c r="C294" s="16" t="inlineStr">
         <is>
-          <t>ILB</t>
-        </is>
-      </c>
-      <c r="D294" s="17" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>SS</t>
+        </is>
+      </c>
+      <c r="D294" s="26" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E294" s="16" t="n">
@@ -12299,7 +12299,7 @@
       </c>
       <c r="H294" s="19" t="inlineStr">
         <is>
-          <t>Linebacker and special teams contributor during his professional career.</t>
+          <t>Defensive back and linebacker who spent time with multiple NFL organizations.</t>
         </is>
       </c>
     </row>
@@ -12309,21 +12309,21 @@
       </c>
       <c r="B295" s="21" t="inlineStr">
         <is>
-          <t>Vadal Alexander</t>
+          <t>Obi Melifonwu</t>
         </is>
       </c>
       <c r="C295" s="22" t="inlineStr">
         <is>
-          <t>OG</t>
-        </is>
-      </c>
-      <c r="D295" s="23" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>SS</t>
+        </is>
+      </c>
+      <c r="D295" s="27" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E295" s="22" t="n">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="F295" s="23" t="inlineStr">
         <is>
@@ -12337,7 +12337,7 @@
       </c>
       <c r="H295" s="25" t="inlineStr">
         <is>
-          <t>Offensive lineman who provided depth during his NFL career.</t>
+          <t>Defensive back whose NFL career was limited by injuries.</t>
         </is>
       </c>
     </row>
@@ -12347,12 +12347,12 @@
       </c>
       <c r="B296" s="15" t="inlineStr">
         <is>
-          <t>Jeremy Cash</t>
+          <t>Caleb Brantley</t>
         </is>
       </c>
       <c r="C296" s="16" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="D296" s="26" t="inlineStr">
@@ -12361,7 +12361,7 @@
         </is>
       </c>
       <c r="E296" s="16" t="n">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="F296" s="26" t="inlineStr">
         <is>
@@ -12375,7 +12375,7 @@
       </c>
       <c r="H296" s="19" t="inlineStr">
         <is>
-          <t>Defensive back and linebacker who spent time with multiple NFL organizations.</t>
+          <t>Defensive lineman whose NFL career was brief.</t>
         </is>
       </c>
     </row>
@@ -12385,12 +12385,12 @@
       </c>
       <c r="B297" s="21" t="inlineStr">
         <is>
-          <t>Caleb Brantley</t>
+          <t>Kendell Beckwith</t>
         </is>
       </c>
       <c r="C297" s="22" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>ILB</t>
         </is>
       </c>
       <c r="D297" s="23" t="inlineStr">
@@ -12413,7 +12413,7 @@
       </c>
       <c r="H297" s="25" t="inlineStr">
         <is>
-          <t>Defensive lineman whose NFL career was brief.</t>
+          <t>Linebacker whose NFL career was shortened by injury.</t>
         </is>
       </c>
     </row>
@@ -12423,21 +12423,21 @@
       </c>
       <c r="B298" s="15" t="inlineStr">
         <is>
-          <t>Kendell Beckwith</t>
+          <t>Jace Sternberger</t>
         </is>
       </c>
       <c r="C298" s="16" t="inlineStr">
         <is>
-          <t>ILB</t>
-        </is>
-      </c>
-      <c r="D298" s="26" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>TE</t>
+        </is>
+      </c>
+      <c r="D298" s="17" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E298" s="16" t="n">
-        <v>2017</v>
+        <v>2019</v>
       </c>
       <c r="F298" s="26" t="inlineStr">
         <is>
@@ -12451,7 +12451,7 @@
       </c>
       <c r="H298" s="19" t="inlineStr">
         <is>
-          <t>Linebacker whose NFL career was shortened by injury.</t>
+          <t>Tight end who spent time in the NFL and alternative professional leagues.</t>
         </is>
       </c>
     </row>
@@ -12461,12 +12461,12 @@
       </c>
       <c r="B299" s="21" t="inlineStr">
         <is>
-          <t>Jace Sternberger</t>
+          <t>Deandre Baker</t>
         </is>
       </c>
       <c r="C299" s="22" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D299" s="27" t="inlineStr">
@@ -12489,7 +12489,7 @@
       </c>
       <c r="H299" s="25" t="inlineStr">
         <is>
-          <t>Tight end who spent time in the NFL and alternative professional leagues.</t>
+          <t>Cornerback whose NFL career was limited by injuries and availability issues.</t>
         </is>
       </c>
     </row>
@@ -12499,25 +12499,25 @@
       </c>
       <c r="B300" s="15" t="inlineStr">
         <is>
-          <t>Tyree Gillespie</t>
+          <t>Jake Fisher</t>
         </is>
       </c>
       <c r="C300" s="16" t="inlineStr">
         <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="D300" s="17" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="D300" s="26" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E300" s="16" t="n">
-        <v>2021</v>
+        <v>2015</v>
       </c>
       <c r="F300" s="26" t="inlineStr">
         <is>
-          <t>29.5</t>
+          <t>28.0</t>
         </is>
       </c>
       <c r="G300" s="26" t="inlineStr">
@@ -12527,7 +12527,7 @@
       </c>
       <c r="H300" s="19" t="inlineStr">
         <is>
-          <t>Safety who spent time with multiple NFL organizations; Super Bowl champion. [PFR correction — SB Win 0→1.]</t>
+          <t>Offensive lineman who provided depth across multiple NFL teams.</t>
         </is>
       </c>
     </row>
@@ -12537,21 +12537,21 @@
       </c>
       <c r="B301" s="21" t="inlineStr">
         <is>
-          <t>Jake Fisher</t>
+          <t>Malik McDowell</t>
         </is>
       </c>
       <c r="C301" s="22" t="inlineStr">
         <is>
-          <t>OT</t>
-        </is>
-      </c>
-      <c r="D301" s="23" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="D301" s="27" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E301" s="22" t="n">
-        <v>2015</v>
+        <v>2017</v>
       </c>
       <c r="F301" s="23" t="inlineStr">
         <is>
@@ -12565,7 +12565,7 @@
       </c>
       <c r="H301" s="25" t="inlineStr">
         <is>
-          <t>Offensive lineman who provided depth across multiple NFL teams.</t>
+          <t>Defensive lineman whose NFL career was derailed early by injuries and off-field issues.</t>
         </is>
       </c>
     </row>
@@ -12575,12 +12575,12 @@
       </c>
       <c r="B302" s="15" t="inlineStr">
         <is>
-          <t>Malik McDowell</t>
+          <t>Holton Hill</t>
         </is>
       </c>
       <c r="C302" s="16" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D302" s="17" t="inlineStr">
@@ -12589,7 +12589,7 @@
         </is>
       </c>
       <c r="E302" s="16" t="n">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="F302" s="26" t="inlineStr">
         <is>
@@ -12603,7 +12603,7 @@
       </c>
       <c r="H302" s="19" t="inlineStr">
         <is>
-          <t>Defensive lineman whose NFL career was derailed early by injuries and off-field issues.</t>
+          <t>Cornerback whose NFL career was limited by injuries and suspensions.</t>
         </is>
       </c>
     </row>
@@ -12613,17 +12613,17 @@
       </c>
       <c r="B303" s="21" t="inlineStr">
         <is>
-          <t>Holton Hill</t>
+          <t>Malik Jefferson</t>
         </is>
       </c>
       <c r="C303" s="22" t="inlineStr">
         <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="D303" s="27" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>OLB</t>
+        </is>
+      </c>
+      <c r="D303" s="23" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E303" s="22" t="n">
@@ -12641,7 +12641,7 @@
       </c>
       <c r="H303" s="25" t="inlineStr">
         <is>
-          <t>Cornerback whose NFL career was limited by injuries and suspensions.</t>
+          <t>Linebacker whose NFL career was primarily spent in reserve roles.</t>
         </is>
       </c>
     </row>
@@ -12651,21 +12651,21 @@
       </c>
       <c r="B304" s="15" t="inlineStr">
         <is>
-          <t>Malik Jefferson</t>
+          <t>Tre Lamar</t>
         </is>
       </c>
       <c r="C304" s="16" t="inlineStr">
         <is>
-          <t>OLB</t>
-        </is>
-      </c>
-      <c r="D304" s="26" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="D304" s="17" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E304" s="16" t="n">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="F304" s="26" t="inlineStr">
         <is>
@@ -12679,7 +12679,7 @@
       </c>
       <c r="H304" s="19" t="inlineStr">
         <is>
-          <t>Linebacker whose NFL career was primarily spent in reserve roles.</t>
+          <t>Linebacker who spent time on NFL rosters and practice squads.</t>
         </is>
       </c>
     </row>
@@ -12689,17 +12689,17 @@
       </c>
       <c r="B305" s="21" t="inlineStr">
         <is>
-          <t>Tre Lamar</t>
+          <t>Elijah Holyfield</t>
         </is>
       </c>
       <c r="C305" s="22" t="inlineStr">
         <is>
-          <t>LB</t>
-        </is>
-      </c>
-      <c r="D305" s="27" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>RB</t>
+        </is>
+      </c>
+      <c r="D305" s="23" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E305" s="22" t="n">
@@ -12717,7 +12717,7 @@
       </c>
       <c r="H305" s="25" t="inlineStr">
         <is>
-          <t>Linebacker who spent time on NFL rosters and practice squads.</t>
+          <t>Running back who spent time with multiple NFL organizations.</t>
         </is>
       </c>
     </row>
@@ -12727,12 +12727,12 @@
       </c>
       <c r="B306" s="15" t="inlineStr">
         <is>
-          <t>Elijah Holyfield</t>
+          <t>Chase Winovich</t>
         </is>
       </c>
       <c r="C306" s="16" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>EDGE</t>
         </is>
       </c>
       <c r="D306" s="26" t="inlineStr">
@@ -12755,7 +12755,7 @@
       </c>
       <c r="H306" s="19" t="inlineStr">
         <is>
-          <t>Running back who spent time with multiple NFL organizations.</t>
+          <t>Edge rusher who contributed as a starter and rotational defender.</t>
         </is>
       </c>
     </row>
@@ -12765,12 +12765,12 @@
       </c>
       <c r="B307" s="21" t="inlineStr">
         <is>
-          <t>Chase Winovich</t>
+          <t>Thaddeus Moss</t>
         </is>
       </c>
       <c r="C307" s="22" t="inlineStr">
         <is>
-          <t>EDGE</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D307" s="23" t="inlineStr">
@@ -12779,7 +12779,7 @@
         </is>
       </c>
       <c r="E307" s="22" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="F307" s="23" t="inlineStr">
         <is>
@@ -12793,7 +12793,7 @@
       </c>
       <c r="H307" s="25" t="inlineStr">
         <is>
-          <t>Edge rusher who contributed as a starter and rotational defender.</t>
+          <t>Tight end who spent time with NFL organizations following a standout college career.</t>
         </is>
       </c>
     </row>
@@ -12803,21 +12803,21 @@
       </c>
       <c r="B308" s="15" t="inlineStr">
         <is>
-          <t>Thaddeus Moss</t>
+          <t>Alex Leatherwood</t>
         </is>
       </c>
       <c r="C308" s="16" t="inlineStr">
         <is>
-          <t>TE</t>
-        </is>
-      </c>
-      <c r="D308" s="26" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>OL</t>
+        </is>
+      </c>
+      <c r="D308" s="17" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E308" s="16" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="F308" s="26" t="inlineStr">
         <is>
@@ -12831,7 +12831,7 @@
       </c>
       <c r="H308" s="19" t="inlineStr">
         <is>
-          <t>Tight end who spent time with NFL organizations following a standout college career.</t>
+          <t>Offensive lineman who spent time with multiple NFL organizations.</t>
         </is>
       </c>
     </row>
@@ -12841,12 +12841,12 @@
       </c>
       <c r="B309" s="21" t="inlineStr">
         <is>
-          <t>Alex Leatherwood</t>
+          <t>Wyatt Hubert</t>
         </is>
       </c>
       <c r="C309" s="22" t="inlineStr">
         <is>
-          <t>OL</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D309" s="27" t="inlineStr">
@@ -12869,7 +12869,7 @@
       </c>
       <c r="H309" s="25" t="inlineStr">
         <is>
-          <t>Offensive lineman who spent time with multiple NFL organizations.</t>
+          <t>Defender whose professional career was limited by injuries.</t>
         </is>
       </c>
     </row>
@@ -12879,12 +12879,12 @@
       </c>
       <c r="B310" s="15" t="inlineStr">
         <is>
-          <t>Wyatt Hubert</t>
+          <t>Tyree Gillespie</t>
         </is>
       </c>
       <c r="C310" s="16" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D310" s="17" t="inlineStr">
@@ -12907,7 +12907,7 @@
       </c>
       <c r="H310" s="19" t="inlineStr">
         <is>
-          <t>Defender whose professional career was limited by injuries.</t>
+          <t>Safety who spent time with multiple NFL organizations.</t>
         </is>
       </c>
     </row>
@@ -13135,7 +13135,7 @@
       </c>
       <c r="H316" s="19" t="inlineStr">
         <is>
-          <t>Offensive lineman whose NFL career was limited by injuries; Super Bowl champion. [PFR correction — SB Win 0→1.]</t>
+          <t>Offensive lineman whose NFL career was limited by injuries.; Super Bowl LI champion with the Patriots. [PFR correction — SB Win 0→1.]</t>
         </is>
       </c>
     </row>
@@ -14691,12 +14691,12 @@
       </c>
       <c r="C5" s="36" t="inlineStr">
         <is>
-          <t>54.32</t>
+          <t>54.24</t>
         </is>
       </c>
       <c r="D5" s="37" t="inlineStr">
         <is>
-          <t>60.03</t>
+          <t>59.98</t>
         </is>
       </c>
       <c r="E5" s="37" t="inlineStr">
@@ -14823,12 +14823,12 @@
       </c>
       <c r="C11" s="36" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>26</t>
         </is>
       </c>
       <c r="D11" s="37" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>18</t>
         </is>
       </c>
       <c r="E11" s="36" t="inlineStr">
@@ -14850,7 +14850,7 @@
       </c>
       <c r="D12" s="33" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>40</t>
         </is>
       </c>
       <c r="E12" s="33" t="inlineStr">

</xml_diff>

<commit_message>
Award gap fixes (RG III/Chase/Lamb/Melifonwu/Haynes) in workbooks
</commit_message>
<xml_diff>
--- a/Trail_Bish_Dynasty_Premium.xlsx
+++ b/Trail_Bish_Dynasty_Premium.xlsx
@@ -884,7 +884,7 @@
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>avg 54.2</t>
+          <t>avg 54.3</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
@@ -1821,25 +1821,25 @@
       </c>
       <c r="B19" s="21" t="inlineStr">
         <is>
-          <t>Micah Parsons</t>
+          <t>Ceedee Lamb</t>
         </is>
       </c>
       <c r="C19" s="22" t="inlineStr">
         <is>
-          <t>LB</t>
-        </is>
-      </c>
-      <c r="D19" s="27" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>WR</t>
+        </is>
+      </c>
+      <c r="D19" s="23" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E19" s="22" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="F19" s="27" t="inlineStr">
         <is>
-          <t>85.1</t>
+          <t>85.5</t>
         </is>
       </c>
       <c r="G19" s="27" t="inlineStr">
@@ -1849,7 +1849,7 @@
       </c>
       <c r="H19" s="25" t="inlineStr">
         <is>
-          <t>Multiple All-Pro linebacker and one of the NFL's premier defensive players.</t>
+          <t>Multiple Pro Bowl and All-Pro receiver with several 1,000-yard seasons.</t>
         </is>
       </c>
     </row>
@@ -1859,12 +1859,12 @@
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>Marlon Humphrey</t>
+          <t>Micah Parsons</t>
         </is>
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D20" s="17" t="inlineStr">
@@ -1873,11 +1873,11 @@
         </is>
       </c>
       <c r="E20" s="16" t="n">
-        <v>2017</v>
+        <v>2021</v>
       </c>
       <c r="F20" s="17" t="inlineStr">
         <is>
-          <t>85.0</t>
+          <t>85.1</t>
         </is>
       </c>
       <c r="G20" s="17" t="inlineStr">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="H20" s="19" t="inlineStr">
         <is>
-          <t>Multiple Pro Bowl and All-Pro cornerback; cornerstone of the Ravens secondary.</t>
+          <t>Multiple All-Pro linebacker and one of the NFL's premier defensive players.</t>
         </is>
       </c>
     </row>
@@ -1897,17 +1897,17 @@
       </c>
       <c r="B21" s="21" t="inlineStr">
         <is>
-          <t>Budda Baker</t>
+          <t>Marlon Humphrey</t>
         </is>
       </c>
       <c r="C21" s="22" t="inlineStr">
         <is>
-          <t>FS</t>
-        </is>
-      </c>
-      <c r="D21" s="23" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="D21" s="27" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E21" s="22" t="n">
@@ -1925,7 +1925,7 @@
       </c>
       <c r="H21" s="25" t="inlineStr">
         <is>
-          <t>Multiple All-Pro and Pro Bowl safety; cornerstone defensive player.</t>
+          <t>Multiple Pro Bowl and All-Pro cornerback; cornerstone of the Ravens secondary.</t>
         </is>
       </c>
     </row>
@@ -1935,12 +1935,12 @@
       </c>
       <c r="B22" s="15" t="inlineStr">
         <is>
-          <t>Chris Lindstrom</t>
+          <t>Budda Baker</t>
         </is>
       </c>
       <c r="C22" s="16" t="inlineStr">
         <is>
-          <t>OL</t>
+          <t>FS</t>
         </is>
       </c>
       <c r="D22" s="26" t="inlineStr">
@@ -1949,11 +1949,11 @@
         </is>
       </c>
       <c r="E22" s="16" t="n">
-        <v>2019</v>
+        <v>2017</v>
       </c>
       <c r="F22" s="17" t="inlineStr">
         <is>
-          <t>84.0</t>
+          <t>85.0</t>
         </is>
       </c>
       <c r="G22" s="17" t="inlineStr">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="H22" s="19" t="inlineStr">
         <is>
-          <t>Multiple All-Pro and Pro Bowl guard; among the NFL's premier interior linemen.</t>
+          <t>Multiple All-Pro and Pro Bowl safety; cornerstone defensive player.</t>
         </is>
       </c>
     </row>
@@ -1973,12 +1973,12 @@
       </c>
       <c r="B23" s="21" t="inlineStr">
         <is>
-          <t>Ceedee Lamb</t>
+          <t>Chris Lindstrom</t>
         </is>
       </c>
       <c r="C23" s="22" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>OL</t>
         </is>
       </c>
       <c r="D23" s="23" t="inlineStr">
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="E23" s="22" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="F23" s="27" t="inlineStr">
         <is>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="H23" s="25" t="inlineStr">
         <is>
-          <t>Multiple Pro Bowl and All-Pro receiver with several 1,000-yard seasons.</t>
+          <t>Multiple All-Pro and Pro Bowl guard; among the NFL's premier interior linemen.</t>
         </is>
       </c>
     </row>
@@ -2011,12 +2011,12 @@
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>Sauce Gardner</t>
+          <t>Ja'marr Chase</t>
         </is>
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D24" s="26" t="inlineStr">
@@ -2025,7 +2025,7 @@
         </is>
       </c>
       <c r="E24" s="16" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F24" s="17" t="inlineStr">
         <is>
@@ -2039,7 +2039,7 @@
       </c>
       <c r="H24" s="19" t="inlineStr">
         <is>
-          <t>Multiple All-Pro cornerback and one of the NFL's premier coverage defenders.</t>
+          <t>Multiple Pro Bowl and All-Pro receiver; among the league's most productive pass catchers.</t>
         </is>
       </c>
     </row>
@@ -2049,25 +2049,25 @@
       </c>
       <c r="B25" s="21" t="inlineStr">
         <is>
-          <t>Ryan Ramczyk</t>
+          <t>Sauce Gardner</t>
         </is>
       </c>
       <c r="C25" s="22" t="inlineStr">
         <is>
-          <t>OT</t>
-        </is>
-      </c>
-      <c r="D25" s="27" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="D25" s="23" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E25" s="22" t="n">
-        <v>2017</v>
+        <v>2022</v>
       </c>
       <c r="F25" s="27" t="inlineStr">
         <is>
-          <t>83.5</t>
+          <t>83.6</t>
         </is>
       </c>
       <c r="G25" s="27" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="H25" s="25" t="inlineStr">
         <is>
-          <t>Multiple All-Pro and Pro Bowl offensive tackle; cornerstone of the Saints offensive line.</t>
+          <t>Multiple All-Pro cornerback and one of the NFL's premier coverage defenders.</t>
         </is>
       </c>
     </row>
@@ -2087,25 +2087,25 @@
       </c>
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>Joey Bosa</t>
+          <t>Ryan Ramczyk</t>
         </is>
       </c>
       <c r="C26" s="16" t="inlineStr">
         <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D26" s="26" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E26" s="16" t="n">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="F26" s="17" t="inlineStr">
         <is>
-          <t>82.6</t>
+          <t>83.5</t>
         </is>
       </c>
       <c r="G26" s="17" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="H26" s="19" t="inlineStr">
         <is>
-          <t>Multiple Pro Bowl pass rusher with over 70 career sacks.</t>
+          <t>Multiple All-Pro and Pro Bowl offensive tackle; cornerstone of the Saints offensive line.</t>
         </is>
       </c>
     </row>
@@ -2125,12 +2125,12 @@
       </c>
       <c r="B27" s="21" t="inlineStr">
         <is>
-          <t>Marshon Lattimore</t>
+          <t>Joey Bosa</t>
         </is>
       </c>
       <c r="C27" s="22" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D27" s="23" t="inlineStr">
@@ -2139,7 +2139,7 @@
         </is>
       </c>
       <c r="E27" s="22" t="n">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="F27" s="27" t="inlineStr">
         <is>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="H27" s="25" t="inlineStr">
         <is>
-          <t>DROY winner and multiple Pro Bowl cornerback.</t>
+          <t>Multiple Pro Bowl pass rusher with over 70 career sacks.</t>
         </is>
       </c>
     </row>
@@ -2163,12 +2163,12 @@
       </c>
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>Roquan Smith</t>
+          <t>Marshon Lattimore</t>
         </is>
       </c>
       <c r="C28" s="16" t="inlineStr">
         <is>
-          <t>ILB</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="D28" s="26" t="inlineStr">
@@ -2177,11 +2177,11 @@
         </is>
       </c>
       <c r="E28" s="16" t="n">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="F28" s="17" t="inlineStr">
         <is>
-          <t>82.5</t>
+          <t>82.6</t>
         </is>
       </c>
       <c r="G28" s="17" t="inlineStr">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="H28" s="19" t="inlineStr">
         <is>
-          <t>Multiple All-Pro linebacker and one of the NFL's leading tacklers.</t>
+          <t>DROY winner and multiple Pro Bowl cornerback.</t>
         </is>
       </c>
     </row>
@@ -2201,12 +2201,12 @@
       </c>
       <c r="B29" s="21" t="inlineStr">
         <is>
-          <t>Amari Cooper</t>
+          <t>Roquan Smith</t>
         </is>
       </c>
       <c r="C29" s="22" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>ILB</t>
         </is>
       </c>
       <c r="D29" s="23" t="inlineStr">
@@ -2215,11 +2215,11 @@
         </is>
       </c>
       <c r="E29" s="22" t="n">
-        <v>2015</v>
+        <v>2018</v>
       </c>
       <c r="F29" s="27" t="inlineStr">
         <is>
-          <t>82.0</t>
+          <t>82.5</t>
         </is>
       </c>
       <c r="G29" s="27" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="H29" s="25" t="inlineStr">
         <is>
-          <t>Multiple Pro Bowl receiver with seven 1,000-yard receiving seasons.</t>
+          <t>Multiple All-Pro linebacker and one of the NFL's leading tacklers.</t>
         </is>
       </c>
     </row>
@@ -2239,12 +2239,12 @@
       </c>
       <c r="B30" s="15" t="inlineStr">
         <is>
-          <t>Laremy Tunsil</t>
+          <t>Amari Cooper</t>
         </is>
       </c>
       <c r="C30" s="16" t="inlineStr">
         <is>
-          <t>OT</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D30" s="26" t="inlineStr">
@@ -2253,7 +2253,7 @@
         </is>
       </c>
       <c r="E30" s="16" t="n">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="F30" s="17" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
       </c>
       <c r="H30" s="19" t="inlineStr">
         <is>
-          <t>Multiple All-Pro and Pro Bowl offensive tackle; among the league's premier pass protectors.</t>
+          <t>Multiple Pro Bowl receiver with seven 1,000-yard receiving seasons.</t>
         </is>
       </c>
     </row>
@@ -2277,21 +2277,21 @@
       </c>
       <c r="B31" s="21" t="inlineStr">
         <is>
-          <t>Jonathan Allen</t>
+          <t>Laremy Tunsil</t>
         </is>
       </c>
       <c r="C31" s="22" t="inlineStr">
         <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D31" s="27" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="D31" s="23" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E31" s="22" t="n">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="F31" s="27" t="inlineStr">
         <is>
@@ -2305,7 +2305,7 @@
       </c>
       <c r="H31" s="25" t="inlineStr">
         <is>
-          <t>Multiple Pro Bowl defensive lineman and key contributor on playoff teams.</t>
+          <t>Multiple All-Pro and Pro Bowl offensive tackle; among the league's premier pass protectors.</t>
         </is>
       </c>
     </row>
@@ -2315,17 +2315,17 @@
       </c>
       <c r="B32" s="15" t="inlineStr">
         <is>
-          <t>Leonard Fournette</t>
+          <t>Jonathan Allen</t>
         </is>
       </c>
       <c r="C32" s="16" t="inlineStr">
         <is>
-          <t>RB</t>
-        </is>
-      </c>
-      <c r="D32" s="26" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D32" s="17" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E32" s="16" t="n">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="F32" s="17" t="inlineStr">
         <is>
-          <t>81.5</t>
+          <t>82.0</t>
         </is>
       </c>
       <c r="G32" s="17" t="inlineStr">
@@ -2343,7 +2343,7 @@
       </c>
       <c r="H32" s="19" t="inlineStr">
         <is>
-          <t>Pro Bowl running back and Super Bowl champion with multiple 1,000-yard seasons.</t>
+          <t>Multiple Pro Bowl defensive lineman and key contributor on playoff teams.</t>
         </is>
       </c>
     </row>
@@ -2353,12 +2353,12 @@
       </c>
       <c r="B33" s="21" t="inlineStr">
         <is>
-          <t>Jalen Carter</t>
+          <t>Leonard Fournette</t>
         </is>
       </c>
       <c r="C33" s="22" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="D33" s="23" t="inlineStr">
@@ -2367,7 +2367,7 @@
         </is>
       </c>
       <c r="E33" s="22" t="n">
-        <v>2023</v>
+        <v>2017</v>
       </c>
       <c r="F33" s="27" t="inlineStr">
         <is>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="H33" s="25" t="inlineStr">
         <is>
-          <t>Pro Bowl defensive tackle and key contributor on elite defenses.</t>
+          <t>Pro Bowl running back and Super Bowl champion with multiple 1,000-yard seasons.</t>
         </is>
       </c>
     </row>
@@ -2391,12 +2391,12 @@
       </c>
       <c r="B34" s="15" t="inlineStr">
         <is>
-          <t>Andrew Luck</t>
+          <t>Jalen Carter</t>
         </is>
       </c>
       <c r="C34" s="16" t="inlineStr">
         <is>
-          <t>QB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D34" s="26" t="inlineStr">
@@ -2405,11 +2405,11 @@
         </is>
       </c>
       <c r="E34" s="16" t="n">
-        <v>2012</v>
+        <v>2023</v>
       </c>
       <c r="F34" s="17" t="inlineStr">
         <is>
-          <t>80.0</t>
+          <t>81.5</t>
         </is>
       </c>
       <c r="G34" s="17" t="inlineStr">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="H34" s="19" t="inlineStr">
         <is>
-          <t>Four-time Pro Bowl franchise QB with multiple elite seasons and major organizational impact.</t>
+          <t>Pro Bowl defensive tackle and key contributor on elite defenses.</t>
         </is>
       </c>
     </row>
@@ -2429,12 +2429,12 @@
       </c>
       <c r="B35" s="21" t="inlineStr">
         <is>
-          <t>Ja'marr Chase</t>
+          <t>Andrew Luck</t>
         </is>
       </c>
       <c r="C35" s="22" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D35" s="23" t="inlineStr">
@@ -2443,7 +2443,7 @@
         </is>
       </c>
       <c r="E35" s="22" t="n">
-        <v>2021</v>
+        <v>2012</v>
       </c>
       <c r="F35" s="27" t="inlineStr">
         <is>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="H35" s="25" t="inlineStr">
         <is>
-          <t>Multiple Pro Bowl and All-Pro receiver; among the league's most productive pass catchers.</t>
+          <t>Four-time Pro Bowl franchise QB with multiple elite seasons and major organizational impact.</t>
         </is>
       </c>
     </row>
@@ -7635,12 +7635,12 @@
       </c>
       <c r="B172" s="15" t="inlineStr">
         <is>
-          <t>Deon Bush</t>
+          <t>Christian Haynes</t>
         </is>
       </c>
       <c r="C172" s="16" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>OL</t>
         </is>
       </c>
       <c r="D172" s="17" t="inlineStr">
@@ -7649,11 +7649,11 @@
         </is>
       </c>
       <c r="E172" s="16" t="n">
-        <v>2016</v>
+        <v>2024</v>
       </c>
       <c r="F172" s="14" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>55.5</t>
         </is>
       </c>
       <c r="G172" s="14" t="inlineStr">
@@ -7663,7 +7663,7 @@
       </c>
       <c r="H172" s="19" t="inlineStr">
         <is>
-          <t>Super Bowl champion safety and long-term depth contributor.</t>
+          <t>Interior offensive lineman with starting potential and early NFL experience.; Super Bowl champion — clipboard ring (scores in v1, zeroed in v2.1 model). [PFR correction — SB Win 0→1.]</t>
         </is>
       </c>
     </row>
@@ -7673,12 +7673,12 @@
       </c>
       <c r="B173" s="21" t="inlineStr">
         <is>
-          <t>Jesse James</t>
+          <t>Deon Bush</t>
         </is>
       </c>
       <c r="C173" s="22" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>SS</t>
         </is>
       </c>
       <c r="D173" s="27" t="inlineStr">
@@ -7687,11 +7687,11 @@
         </is>
       </c>
       <c r="E173" s="22" t="n">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="F173" s="20" t="inlineStr">
         <is>
-          <t>54.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G173" s="20" t="inlineStr">
@@ -7701,7 +7701,7 @@
       </c>
       <c r="H173" s="25" t="inlineStr">
         <is>
-          <t>Long-term NFL tight end and reliable red-zone contributor.</t>
+          <t>Super Bowl champion safety and long-term depth contributor.</t>
         </is>
       </c>
     </row>
@@ -7711,12 +7711,12 @@
       </c>
       <c r="B174" s="15" t="inlineStr">
         <is>
-          <t>Trae Waynes</t>
+          <t>Jesse James</t>
         </is>
       </c>
       <c r="C174" s="16" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D174" s="17" t="inlineStr">
@@ -7739,7 +7739,7 @@
       </c>
       <c r="H174" s="19" t="inlineStr">
         <is>
-          <t>Starting cornerback whose career was impacted by injuries.</t>
+          <t>Long-term NFL tight end and reliable red-zone contributor.</t>
         </is>
       </c>
     </row>
@@ -7749,21 +7749,21 @@
       </c>
       <c r="B175" s="21" t="inlineStr">
         <is>
-          <t>Nick Vannett</t>
+          <t>Trae Waynes</t>
         </is>
       </c>
       <c r="C175" s="22" t="inlineStr">
         <is>
-          <t>TE</t>
-        </is>
-      </c>
-      <c r="D175" s="23" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="D175" s="27" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E175" s="22" t="n">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="F175" s="20" t="inlineStr">
         <is>
@@ -7777,7 +7777,7 @@
       </c>
       <c r="H175" s="25" t="inlineStr">
         <is>
-          <t>Blocking tight end and reliable depth contributor.</t>
+          <t>Starting cornerback whose career was impacted by injuries.</t>
         </is>
       </c>
     </row>
@@ -7787,12 +7787,12 @@
       </c>
       <c r="B176" s="15" t="inlineStr">
         <is>
-          <t>Artie Burns</t>
+          <t>Nick Vannett</t>
         </is>
       </c>
       <c r="C176" s="16" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D176" s="26" t="inlineStr">
@@ -7815,7 +7815,7 @@
       </c>
       <c r="H176" s="19" t="inlineStr">
         <is>
-          <t>Cornerback who contributed as a starter and depth player during his NFL career.</t>
+          <t>Blocking tight end and reliable depth contributor.</t>
         </is>
       </c>
     </row>
@@ -7825,21 +7825,21 @@
       </c>
       <c r="B177" s="21" t="inlineStr">
         <is>
-          <t>Mitchell Trubisky</t>
+          <t>Artie Burns</t>
         </is>
       </c>
       <c r="C177" s="22" t="inlineStr">
         <is>
-          <t>QB</t>
-        </is>
-      </c>
-      <c r="D177" s="27" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="D177" s="23" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E177" s="22" t="n">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="F177" s="20" t="inlineStr">
         <is>
@@ -7853,7 +7853,7 @@
       </c>
       <c r="H177" s="25" t="inlineStr">
         <is>
-          <t>Pro Bowl quarterback who started multiple seasons and led the Bears to a playoff appearance.</t>
+          <t>Cornerback who contributed as a starter and depth player during his NFL career.</t>
         </is>
       </c>
     </row>
@@ -7863,12 +7863,12 @@
       </c>
       <c r="B178" s="15" t="inlineStr">
         <is>
-          <t>Michael Gallup</t>
+          <t>Mitchell Trubisky</t>
         </is>
       </c>
       <c r="C178" s="16" t="inlineStr">
         <is>
-          <t>WR</t>
+          <t>QB</t>
         </is>
       </c>
       <c r="D178" s="17" t="inlineStr">
@@ -7877,7 +7877,7 @@
         </is>
       </c>
       <c r="E178" s="16" t="n">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="F178" s="14" t="inlineStr">
         <is>
@@ -7891,7 +7891,7 @@
       </c>
       <c r="H178" s="19" t="inlineStr">
         <is>
-          <t>Productive starting receiver with multiple 800+ yard seasons.</t>
+          <t>Pro Bowl quarterback who started multiple seasons and led the Bears to a playoff appearance.</t>
         </is>
       </c>
     </row>
@@ -7901,12 +7901,12 @@
       </c>
       <c r="B179" s="21" t="inlineStr">
         <is>
-          <t>Maurice Hurst Jr.</t>
+          <t>Michael Gallup</t>
         </is>
       </c>
       <c r="C179" s="22" t="inlineStr">
         <is>
-          <t>DT</t>
+          <t>WR</t>
         </is>
       </c>
       <c r="D179" s="27" t="inlineStr">
@@ -7929,7 +7929,7 @@
       </c>
       <c r="H179" s="25" t="inlineStr">
         <is>
-          <t>Defensive tackle who contributed as a rotational starter and depth player.</t>
+          <t>Productive starting receiver with multiple 800+ yard seasons.</t>
         </is>
       </c>
     </row>
@@ -7939,21 +7939,21 @@
       </c>
       <c r="B180" s="15" t="inlineStr">
         <is>
-          <t>Teven Jenkins</t>
+          <t>Maurice Hurst Jr.</t>
         </is>
       </c>
       <c r="C180" s="16" t="inlineStr">
         <is>
-          <t>OL</t>
-        </is>
-      </c>
-      <c r="D180" s="26" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>DT</t>
+        </is>
+      </c>
+      <c r="D180" s="17" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E180" s="16" t="n">
-        <v>2021</v>
+        <v>2018</v>
       </c>
       <c r="F180" s="14" t="inlineStr">
         <is>
@@ -7967,7 +7967,7 @@
       </c>
       <c r="H180" s="19" t="inlineStr">
         <is>
-          <t>Starting offensive lineman known for versatility and physical play.</t>
+          <t>Defensive tackle who contributed as a rotational starter and depth player.</t>
         </is>
       </c>
     </row>
@@ -7977,12 +7977,12 @@
       </c>
       <c r="B181" s="21" t="inlineStr">
         <is>
-          <t>Malcolm Koonce</t>
+          <t>Teven Jenkins</t>
         </is>
       </c>
       <c r="C181" s="22" t="inlineStr">
         <is>
-          <t>EDGE</t>
+          <t>OL</t>
         </is>
       </c>
       <c r="D181" s="23" t="inlineStr">
@@ -8005,7 +8005,7 @@
       </c>
       <c r="H181" s="25" t="inlineStr">
         <is>
-          <t>Edge rusher who developed into a productive defensive contributor.</t>
+          <t>Starting offensive lineman known for versatility and physical play.</t>
         </is>
       </c>
     </row>
@@ -8015,12 +8015,12 @@
       </c>
       <c r="B182" s="15" t="inlineStr">
         <is>
-          <t>Zaven Collins</t>
+          <t>Malcolm Koonce</t>
         </is>
       </c>
       <c r="C182" s="16" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>EDGE</t>
         </is>
       </c>
       <c r="D182" s="26" t="inlineStr">
@@ -8043,7 +8043,7 @@
       </c>
       <c r="H182" s="19" t="inlineStr">
         <is>
-          <t>Linebacker and defensive contributor with starting experience.</t>
+          <t>Edge rusher who developed into a productive defensive contributor.</t>
         </is>
       </c>
     </row>
@@ -8053,7 +8053,7 @@
       </c>
       <c r="B183" s="21" t="inlineStr">
         <is>
-          <t>Isaiah Mcduffie</t>
+          <t>Zaven Collins</t>
         </is>
       </c>
       <c r="C183" s="22" t="inlineStr">
@@ -8081,7 +8081,7 @@
       </c>
       <c r="H183" s="25" t="inlineStr">
         <is>
-          <t>Linebacker and special teams contributor who earned a larger defensive role.</t>
+          <t>Linebacker and defensive contributor with starting experience.</t>
         </is>
       </c>
     </row>
@@ -8091,12 +8091,12 @@
       </c>
       <c r="B184" s="15" t="inlineStr">
         <is>
-          <t>Caden Sterns</t>
+          <t>Isaiah Mcduffie</t>
         </is>
       </c>
       <c r="C184" s="16" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="D184" s="26" t="inlineStr">
@@ -8119,7 +8119,7 @@
       </c>
       <c r="H184" s="19" t="inlineStr">
         <is>
-          <t>Safety whose career has been impacted by injuries.</t>
+          <t>Linebacker and special teams contributor who earned a larger defensive role.</t>
         </is>
       </c>
     </row>
@@ -8129,21 +8129,21 @@
       </c>
       <c r="B185" s="21" t="inlineStr">
         <is>
-          <t>Chig Okonkwo</t>
+          <t>Caden Sterns</t>
         </is>
       </c>
       <c r="C185" s="22" t="inlineStr">
         <is>
-          <t>TE</t>
-        </is>
-      </c>
-      <c r="D185" s="27" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D185" s="23" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E185" s="22" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="F185" s="20" t="inlineStr">
         <is>
@@ -8157,7 +8157,7 @@
       </c>
       <c r="H185" s="25" t="inlineStr">
         <is>
-          <t>Athletic tight end and productive receiving contributor.</t>
+          <t>Safety whose career has been impacted by injuries.</t>
         </is>
       </c>
     </row>
@@ -8167,12 +8167,12 @@
       </c>
       <c r="B186" s="15" t="inlineStr">
         <is>
-          <t>Daxton Hill</t>
+          <t>Chig Okonkwo</t>
         </is>
       </c>
       <c r="C186" s="16" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D186" s="17" t="inlineStr">
@@ -8195,7 +8195,7 @@
       </c>
       <c r="H186" s="19" t="inlineStr">
         <is>
-          <t>Defensive back with starting experience in the secondary.</t>
+          <t>Athletic tight end and productive receiving contributor.</t>
         </is>
       </c>
     </row>
@@ -8205,12 +8205,12 @@
       </c>
       <c r="B187" s="21" t="inlineStr">
         <is>
-          <t>Darnell Washington</t>
+          <t>Daxton Hill</t>
         </is>
       </c>
       <c r="C187" s="22" t="inlineStr">
         <is>
-          <t>TE</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D187" s="27" t="inlineStr">
@@ -8219,7 +8219,7 @@
         </is>
       </c>
       <c r="E187" s="22" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="F187" s="20" t="inlineStr">
         <is>
@@ -8233,7 +8233,7 @@
       </c>
       <c r="H187" s="25" t="inlineStr">
         <is>
-          <t>Blocking tight end known for versatility and physical play.</t>
+          <t>Defensive back with starting experience in the secondary.</t>
         </is>
       </c>
     </row>
@@ -8243,12 +8243,12 @@
       </c>
       <c r="B188" s="15" t="inlineStr">
         <is>
-          <t>Sidy Sow</t>
+          <t>Darnell Washington</t>
         </is>
       </c>
       <c r="C188" s="16" t="inlineStr">
         <is>
-          <t>OL</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D188" s="17" t="inlineStr">
@@ -8271,7 +8271,7 @@
       </c>
       <c r="H188" s="19" t="inlineStr">
         <is>
-          <t>Offensive lineman with starting experience and positional versatility.</t>
+          <t>Blocking tight end known for versatility and physical play.</t>
         </is>
       </c>
     </row>
@@ -8281,12 +8281,12 @@
       </c>
       <c r="B189" s="21" t="inlineStr">
         <is>
-          <t>BJ Ojulari</t>
+          <t>Sidy Sow</t>
         </is>
       </c>
       <c r="C189" s="22" t="inlineStr">
         <is>
-          <t>EDGE</t>
+          <t>OL</t>
         </is>
       </c>
       <c r="D189" s="27" t="inlineStr">
@@ -8309,7 +8309,7 @@
       </c>
       <c r="H189" s="25" t="inlineStr">
         <is>
-          <t>Edge defender whose early career has been impacted by injury.</t>
+          <t>Offensive lineman with starting experience and positional versatility.</t>
         </is>
       </c>
     </row>
@@ -8319,12 +8319,12 @@
       </c>
       <c r="B190" s="15" t="inlineStr">
         <is>
-          <t>Mazi Smith</t>
+          <t>BJ Ojulari</t>
         </is>
       </c>
       <c r="C190" s="16" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>EDGE</t>
         </is>
       </c>
       <c r="D190" s="17" t="inlineStr">
@@ -8347,7 +8347,7 @@
       </c>
       <c r="H190" s="19" t="inlineStr">
         <is>
-          <t>Defensive tackle and contributor on the defensive front.</t>
+          <t>Edge defender whose early career has been impacted by injury.</t>
         </is>
       </c>
     </row>
@@ -8357,17 +8357,17 @@
       </c>
       <c r="B191" s="21" t="inlineStr">
         <is>
-          <t>Henry To'oTo'o</t>
+          <t>Mazi Smith</t>
         </is>
       </c>
       <c r="C191" s="22" t="inlineStr">
         <is>
-          <t>LB</t>
-        </is>
-      </c>
-      <c r="D191" s="23" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D191" s="27" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E191" s="22" t="n">
@@ -8385,7 +8385,7 @@
       </c>
       <c r="H191" s="25" t="inlineStr">
         <is>
-          <t>Starting linebacker and productive defensive contributor.</t>
+          <t>Defensive tackle and contributor on the defensive front.</t>
         </is>
       </c>
     </row>
@@ -8395,21 +8395,21 @@
       </c>
       <c r="B192" s="15" t="inlineStr">
         <is>
-          <t>Theo Johnson</t>
+          <t>Henry To'oTo'o</t>
         </is>
       </c>
       <c r="C192" s="16" t="inlineStr">
         <is>
-          <t>TE</t>
-        </is>
-      </c>
-      <c r="D192" s="17" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="D192" s="26" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E192" s="16" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="F192" s="14" t="inlineStr">
         <is>
@@ -8423,7 +8423,7 @@
       </c>
       <c r="H192" s="19" t="inlineStr">
         <is>
-          <t>Athletic tight end and developing receiving target.</t>
+          <t>Starting linebacker and productive defensive contributor.</t>
         </is>
       </c>
     </row>
@@ -8433,12 +8433,12 @@
       </c>
       <c r="B193" s="21" t="inlineStr">
         <is>
-          <t>Christian Haynes</t>
+          <t>Theo Johnson</t>
         </is>
       </c>
       <c r="C193" s="22" t="inlineStr">
         <is>
-          <t>OL</t>
+          <t>TE</t>
         </is>
       </c>
       <c r="D193" s="27" t="inlineStr">
@@ -8461,7 +8461,7 @@
       </c>
       <c r="H193" s="25" t="inlineStr">
         <is>
-          <t>Interior offensive lineman with starting potential and early NFL experience.</t>
+          <t>Athletic tight end and developing receiving target.</t>
         </is>
       </c>
     </row>
@@ -11035,7 +11035,7 @@
       </c>
       <c r="F261" s="22" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>44.6</t>
         </is>
       </c>
       <c r="G261" s="22" t="inlineStr">
@@ -12081,25 +12081,25 @@
       </c>
       <c r="B289" s="21" t="inlineStr">
         <is>
-          <t>Matt Barkley</t>
+          <t>Obi Melifonwu</t>
         </is>
       </c>
       <c r="C289" s="22" t="inlineStr">
         <is>
-          <t>QB</t>
-        </is>
-      </c>
-      <c r="D289" s="23" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>SS</t>
+        </is>
+      </c>
+      <c r="D289" s="27" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E289" s="22" t="n">
-        <v>2013</v>
+        <v>2017</v>
       </c>
       <c r="F289" s="23" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>33.5</t>
         </is>
       </c>
       <c r="G289" s="23" t="inlineStr">
@@ -12109,7 +12109,7 @@
       </c>
       <c r="H289" s="25" t="inlineStr">
         <is>
-          <t>Career backup quarterback who provided depth across multiple organizations.</t>
+          <t>Defensive back whose NFL career was limited by injuries.; Super Bowl champion — clipboard ring (scores in v1, zeroed in v2.1 model). [PFR correction — SB Win 0→1.]</t>
         </is>
       </c>
     </row>
@@ -12119,21 +12119,21 @@
       </c>
       <c r="B290" s="15" t="inlineStr">
         <is>
-          <t>Robert Nkemdiche</t>
+          <t>Matt Barkley</t>
         </is>
       </c>
       <c r="C290" s="16" t="inlineStr">
         <is>
-          <t>DT</t>
-        </is>
-      </c>
-      <c r="D290" s="17" t="inlineStr">
-        <is>
-          <t>Matt</t>
+          <t>QB</t>
+        </is>
+      </c>
+      <c r="D290" s="26" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E290" s="16" t="n">
-        <v>2016</v>
+        <v>2013</v>
       </c>
       <c r="F290" s="26" t="inlineStr">
         <is>
@@ -12147,7 +12147,7 @@
       </c>
       <c r="H290" s="19" t="inlineStr">
         <is>
-          <t>Defensive lineman whose NFL career did not meet first-round expectations.</t>
+          <t>Career backup quarterback who provided depth across multiple organizations.</t>
         </is>
       </c>
     </row>
@@ -12157,12 +12157,12 @@
       </c>
       <c r="B291" s="21" t="inlineStr">
         <is>
-          <t>Kevin Dodd</t>
+          <t>Robert Nkemdiche</t>
         </is>
       </c>
       <c r="C291" s="22" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>DT</t>
         </is>
       </c>
       <c r="D291" s="27" t="inlineStr">
@@ -12185,7 +12185,7 @@
       </c>
       <c r="H291" s="25" t="inlineStr">
         <is>
-          <t>Edge rusher whose NFL career was limited by injuries.</t>
+          <t>Defensive lineman whose NFL career did not meet first-round expectations.</t>
         </is>
       </c>
     </row>
@@ -12195,12 +12195,12 @@
       </c>
       <c r="B292" s="15" t="inlineStr">
         <is>
-          <t>Scooby Wright III</t>
+          <t>Kevin Dodd</t>
         </is>
       </c>
       <c r="C292" s="16" t="inlineStr">
         <is>
-          <t>ILB</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D292" s="17" t="inlineStr">
@@ -12223,7 +12223,7 @@
       </c>
       <c r="H292" s="19" t="inlineStr">
         <is>
-          <t>Linebacker and special teams contributor during his professional career.</t>
+          <t>Edge rusher whose NFL career was limited by injuries.</t>
         </is>
       </c>
     </row>
@@ -12233,17 +12233,17 @@
       </c>
       <c r="B293" s="21" t="inlineStr">
         <is>
-          <t>Vadal Alexander</t>
+          <t>Scooby Wright III</t>
         </is>
       </c>
       <c r="C293" s="22" t="inlineStr">
         <is>
-          <t>OG</t>
-        </is>
-      </c>
-      <c r="D293" s="23" t="inlineStr">
-        <is>
-          <t>Ryan</t>
+          <t>ILB</t>
+        </is>
+      </c>
+      <c r="D293" s="27" t="inlineStr">
+        <is>
+          <t>Matt</t>
         </is>
       </c>
       <c r="E293" s="22" t="n">
@@ -12261,7 +12261,7 @@
       </c>
       <c r="H293" s="25" t="inlineStr">
         <is>
-          <t>Offensive lineman who provided depth during his NFL career.</t>
+          <t>Linebacker and special teams contributor during his professional career.</t>
         </is>
       </c>
     </row>
@@ -12271,12 +12271,12 @@
       </c>
       <c r="B294" s="15" t="inlineStr">
         <is>
-          <t>Jeremy Cash</t>
+          <t>Vadal Alexander</t>
         </is>
       </c>
       <c r="C294" s="16" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>OG</t>
         </is>
       </c>
       <c r="D294" s="26" t="inlineStr">
@@ -12299,7 +12299,7 @@
       </c>
       <c r="H294" s="19" t="inlineStr">
         <is>
-          <t>Defensive back and linebacker who spent time with multiple NFL organizations.</t>
+          <t>Offensive lineman who provided depth during his NFL career.</t>
         </is>
       </c>
     </row>
@@ -12309,7 +12309,7 @@
       </c>
       <c r="B295" s="21" t="inlineStr">
         <is>
-          <t>Obi Melifonwu</t>
+          <t>Jeremy Cash</t>
         </is>
       </c>
       <c r="C295" s="22" t="inlineStr">
@@ -12317,13 +12317,13 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D295" s="27" t="inlineStr">
-        <is>
-          <t>Matt</t>
+      <c r="D295" s="23" t="inlineStr">
+        <is>
+          <t>Ryan</t>
         </is>
       </c>
       <c r="E295" s="22" t="n">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="F295" s="23" t="inlineStr">
         <is>
@@ -12337,7 +12337,7 @@
       </c>
       <c r="H295" s="25" t="inlineStr">
         <is>
-          <t>Defensive back whose NFL career was limited by injuries.</t>
+          <t>Defensive back and linebacker who spent time with multiple NFL organizations.</t>
         </is>
       </c>
     </row>
@@ -14691,12 +14691,12 @@
       </c>
       <c r="C5" s="36" t="inlineStr">
         <is>
-          <t>54.24</t>
+          <t>54.26</t>
         </is>
       </c>
       <c r="D5" s="37" t="inlineStr">
         <is>
-          <t>59.98</t>
+          <t>60.01</t>
         </is>
       </c>
       <c r="E5" s="37" t="inlineStr">
@@ -14823,7 +14823,7 @@
       </c>
       <c r="C11" s="36" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>28</t>
         </is>
       </c>
       <c r="D11" s="37" t="inlineStr">
@@ -14850,7 +14850,7 @@
       </c>
       <c r="D12" s="33" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>43</t>
         </is>
       </c>
       <c r="E12" s="33" t="inlineStr">

</xml_diff>